<commit_message>
Daily attendance processing - 2026-05-18 06:00:56 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>244</v>
+        <v>239</v>
       </c>
     </row>
     <row r="9">
@@ -1289,10 +1289,10 @@
         <v>0</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
@@ -1367,10 +1367,10 @@
         <v>1</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
@@ -1445,10 +1445,10 @@
         <v>0</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
@@ -1523,10 +1523,10 @@
         <v>1</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q18" s="4" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
@@ -1601,10 +1601,10 @@
         <v>1</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
@@ -2457,45 +2457,45 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C38" s="8" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D38" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E38" s="8" t="inlineStr">
         <is>
           <t>18/05/2026</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr"/>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr"/>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -4181,45 +4181,45 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="inlineStr">
+      <c r="A78" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B78" s="8" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr">
+      <c r="C78" s="8" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D78" s="2" t="inlineStr">
+      <c r="D78" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E78" s="2" t="inlineStr">
+      <c r="E78" s="8" t="inlineStr">
         <is>
           <t>18/05/2026</t>
         </is>
       </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="inlineStr"/>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I78" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F78" s="8" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G78" s="8" t="inlineStr"/>
+      <c r="H78" s="8" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I78" s="8" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -5299,45 +5299,45 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B104" s="2" t="inlineStr">
+      <c r="A104" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B104" s="8" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C104" s="2" t="inlineStr">
+      <c r="C104" s="8" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D104" s="2" t="inlineStr">
+      <c r="D104" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E104" s="2" t="inlineStr">
+      <c r="E104" s="8" t="inlineStr">
         <is>
           <t>18/05/2026</t>
         </is>
       </c>
-      <c r="F104" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G104" s="2" t="inlineStr"/>
-      <c r="H104" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I104" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F104" s="8" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G104" s="8" t="inlineStr"/>
+      <c r="H104" s="8" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I104" s="8" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -7840,45 +7840,45 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B163" s="2" t="inlineStr">
+      <c r="A163" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B163" s="8" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C163" s="2" t="inlineStr">
+      <c r="C163" s="8" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D163" s="2" t="inlineStr">
+      <c r="D163" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E163" s="2" t="inlineStr">
+      <c r="E163" s="8" t="inlineStr">
         <is>
           <t>18/05/2026</t>
         </is>
       </c>
-      <c r="F163" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G163" s="2" t="inlineStr"/>
-      <c r="H163" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I163" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F163" s="8" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G163" s="8" t="inlineStr"/>
+      <c r="H163" s="8" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I163" s="8" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -10424,45 +10424,45 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B223" s="2" t="inlineStr">
+      <c r="A223" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B223" s="8" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C223" s="2" t="inlineStr">
+      <c r="C223" s="8" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D223" s="2" t="inlineStr">
+      <c r="D223" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E223" s="2" t="inlineStr">
+      <c r="E223" s="8" t="inlineStr">
         <is>
           <t>18/05/2026</t>
         </is>
       </c>
-      <c r="F223" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G223" s="2" t="inlineStr"/>
-      <c r="H223" s="2" t="inlineStr">
+      <c r="F223" s="8" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G223" s="8" t="inlineStr"/>
+      <c r="H223" s="8" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I223" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I223" s="8" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-30 07:53:25 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="9">
@@ -1445,10 +1445,10 @@
         <v>0</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
@@ -5456,45 +5456,45 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B107" s="2" t="inlineStr">
+      <c r="A107" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B107" s="9" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C107" s="2" t="inlineStr">
+      <c r="C107" s="9" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D107" s="2" t="inlineStr">
+      <c r="D107" s="9" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E107" s="2" t="inlineStr">
+      <c r="E107" s="9" t="inlineStr">
         <is>
           <t>30/05/2026</t>
         </is>
       </c>
-      <c r="F107" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G107" s="2" t="inlineStr"/>
-      <c r="H107" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I107" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F107" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G107" s="9" t="inlineStr"/>
+      <c r="H107" s="9" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I107" s="9" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-31 05:13:53 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>224</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9">
@@ -1289,10 +1289,10 @@
         <v>3</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
@@ -1367,10 +1367,10 @@
         <v>5</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
@@ -1445,10 +1445,10 @@
         <v>0</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
@@ -1523,10 +1523,10 @@
         <v>3</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q18" s="4" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
@@ -1601,10 +1601,10 @@
         <v>5</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
@@ -2641,45 +2641,45 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C42" s="9" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D42" s="9" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E42" s="9" t="inlineStr">
         <is>
           <t>31/05/2026</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr"/>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G42" s="9" t="inlineStr"/>
+      <c r="H42" s="9" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I42" s="9" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -4381,45 +4381,45 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B82" s="2" t="inlineStr">
+      <c r="A82" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B82" s="9" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C82" s="2" t="inlineStr">
+      <c r="C82" s="9" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D82" s="2" t="inlineStr">
+      <c r="D82" s="9" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E82" s="2" t="inlineStr">
+      <c r="E82" s="9" t="inlineStr">
         <is>
           <t>31/05/2026</t>
         </is>
       </c>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G82" s="2" t="inlineStr"/>
-      <c r="H82" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I82" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F82" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G82" s="9" t="inlineStr"/>
+      <c r="H82" s="9" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I82" s="9" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -5499,45 +5499,45 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B108" s="2" t="inlineStr">
+      <c r="A108" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B108" s="9" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C108" s="2" t="inlineStr">
+      <c r="C108" s="9" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D108" s="2" t="inlineStr">
+      <c r="D108" s="9" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E108" s="2" t="inlineStr">
+      <c r="E108" s="9" t="inlineStr">
         <is>
           <t>31/05/2026</t>
         </is>
       </c>
-      <c r="F108" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G108" s="2" t="inlineStr"/>
-      <c r="H108" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I108" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F108" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G108" s="9" t="inlineStr"/>
+      <c r="H108" s="9" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I108" s="9" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -8048,45 +8048,45 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B167" s="2" t="inlineStr">
+      <c r="A167" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B167" s="9" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C167" s="2" t="inlineStr">
+      <c r="C167" s="9" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D167" s="2" t="inlineStr">
+      <c r="D167" s="9" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E167" s="2" t="inlineStr">
+      <c r="E167" s="9" t="inlineStr">
         <is>
           <t>31/05/2026</t>
         </is>
       </c>
-      <c r="F167" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G167" s="2" t="inlineStr"/>
-      <c r="H167" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I167" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F167" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G167" s="9" t="inlineStr"/>
+      <c r="H167" s="9" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I167" s="9" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -11508,45 +11508,45 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B247" s="2" t="inlineStr">
+      <c r="A247" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B247" s="9" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C247" s="2" t="inlineStr">
+      <c r="C247" s="9" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D247" s="2" t="inlineStr">
+      <c r="D247" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E247" s="2" t="inlineStr">
+      <c r="E247" s="9" t="inlineStr">
         <is>
           <t>31/05/2026</t>
         </is>
       </c>
-      <c r="F247" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G247" s="2" t="inlineStr"/>
-      <c r="H247" s="2" t="inlineStr">
+      <c r="F247" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G247" s="9" t="inlineStr"/>
+      <c r="H247" s="9" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I247" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I247" s="9" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-31 17:17:07 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>6.4%</t>
+          <t>6.8%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>71.0%</t>
+          <t>70.7%</t>
         </is>
       </c>
     </row>
@@ -1598,22 +1598,22 @@
         <v>50</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>44</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>67.0%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
@@ -11508,45 +11508,49 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B247" s="9" t="inlineStr">
+      <c r="A247" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B247" s="8" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C247" s="9" t="inlineStr">
+      <c r="C247" s="8" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D247" s="9" t="inlineStr">
+      <c r="D247" s="8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E247" s="9" t="inlineStr">
+      <c r="E247" s="8" t="inlineStr">
         <is>
           <t>31/05/2026</t>
         </is>
       </c>
-      <c r="F247" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G247" s="9" t="inlineStr"/>
-      <c r="H247" s="9" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I247" s="9" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F247" s="8" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G247" s="8" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H247" s="8" t="inlineStr">
+        <is>
+          <t>24/37</t>
+        </is>
+      </c>
+      <c r="I247" s="8" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-06 07:59:06 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="9">
@@ -1367,10 +1367,10 @@
         <v>8</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
@@ -3083,45 +3083,45 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C52" s="9" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="D52" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E52" s="9" t="inlineStr">
         <is>
           <t>06/06/2026</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr"/>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F52" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G52" s="9" t="inlineStr"/>
+      <c r="H52" s="9" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I52" s="9" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-08 14:47:24 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.2%</t>
         </is>
       </c>
     </row>
@@ -1598,22 +1598,22 @@
         <v>50</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>38</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>22.0%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>65.4%</t>
+          <t>65.6%</t>
         </is>
       </c>
     </row>
@@ -11169,45 +11169,49 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B238" s="9" t="inlineStr">
+      <c r="A238" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B238" s="8" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C238" s="9" t="inlineStr">
+      <c r="C238" s="8" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D238" s="9" t="inlineStr">
+      <c r="D238" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E238" s="9" t="inlineStr">
+      <c r="E238" s="8" t="inlineStr">
         <is>
           <t>08/06/2026</t>
         </is>
       </c>
-      <c r="F238" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G238" s="9" t="inlineStr"/>
-      <c r="H238" s="9" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I238" s="9" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F238" s="8" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G238" s="8" t="inlineStr">
+        <is>
+          <t>2027/2028</t>
+        </is>
+      </c>
+      <c r="H238" s="8" t="inlineStr">
+        <is>
+          <t>25/37</t>
+        </is>
+      </c>
+      <c r="I238" s="8" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-10 07:25:20 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="9">
@@ -1289,10 +1289,10 @@
         <v>10</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
@@ -1367,10 +1367,10 @@
         <v>8</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
@@ -1445,10 +1445,10 @@
         <v>1</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
@@ -1523,10 +1523,10 @@
         <v>4</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q18" s="4" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
@@ -1601,10 +1601,10 @@
         <v>12</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
@@ -2125,45 +2125,45 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E30" s="9" t="inlineStr">
         <is>
           <t>10/06/2026</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr"/>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I30" s="9" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -3271,45 +3271,45 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B56" s="9" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C56" s="9" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="D56" s="9" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E56" s="9" t="inlineStr">
         <is>
           <t>10/06/2026</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr"/>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I56" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F56" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G56" s="9" t="inlineStr"/>
+      <c r="H56" s="9" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I56" s="9" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -5844,45 +5844,45 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B115" s="2" t="inlineStr">
+      <c r="A115" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B115" s="9" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C115" s="2" t="inlineStr">
+      <c r="C115" s="9" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D115" s="2" t="inlineStr">
+      <c r="D115" s="9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E115" s="2" t="inlineStr">
+      <c r="E115" s="9" t="inlineStr">
         <is>
           <t>10/06/2026</t>
         </is>
       </c>
-      <c r="F115" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G115" s="2" t="inlineStr"/>
-      <c r="H115" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I115" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F115" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G115" s="9" t="inlineStr"/>
+      <c r="H115" s="9" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I115" s="9" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -8440,45 +8440,45 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B175" s="2" t="inlineStr">
+      <c r="A175" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B175" s="9" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C175" s="2" t="inlineStr">
+      <c r="C175" s="9" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D175" s="2" t="inlineStr">
+      <c r="D175" s="9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E175" s="2" t="inlineStr">
+      <c r="E175" s="9" t="inlineStr">
         <is>
           <t>10/06/2026</t>
         </is>
       </c>
-      <c r="F175" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G175" s="2" t="inlineStr"/>
-      <c r="H175" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I175" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F175" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G175" s="9" t="inlineStr"/>
+      <c r="H175" s="9" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I175" s="9" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -11267,45 +11267,45 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B240" s="2" t="inlineStr">
+      <c r="A240" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B240" s="9" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C240" s="2" t="inlineStr">
+      <c r="C240" s="9" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D240" s="2" t="inlineStr">
+      <c r="D240" s="9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E240" s="2" t="inlineStr">
+      <c r="E240" s="9" t="inlineStr">
         <is>
           <t>10/06/2026</t>
         </is>
       </c>
-      <c r="F240" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G240" s="2" t="inlineStr"/>
-      <c r="H240" s="2" t="inlineStr">
+      <c r="F240" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G240" s="9" t="inlineStr"/>
+      <c r="H240" s="9" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I240" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I240" s="9" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-15 16:04:39 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>16.8%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>65.1%</t>
+          <t>65.6%</t>
         </is>
       </c>
     </row>
@@ -1520,22 +1520,22 @@
         <v>50</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>33</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>45.5%</t>
+          <t>51.1%</t>
         </is>
       </c>
     </row>
@@ -1598,22 +1598,22 @@
         <v>50</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>33</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>26.0%</t>
+          <t>28.0%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>66.9%</t>
+          <t>67.4%</t>
         </is>
       </c>
     </row>
@@ -9445,45 +9445,49 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B198" s="9" t="inlineStr">
+      <c r="A198" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B198" s="8" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C198" s="9" t="inlineStr">
+      <c r="C198" s="8" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D198" s="9" t="inlineStr">
+      <c r="D198" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E198" s="9" t="inlineStr">
+      <c r="E198" s="8" t="inlineStr">
         <is>
           <t>15/06/2026</t>
         </is>
       </c>
-      <c r="F198" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G198" s="9" t="inlineStr"/>
-      <c r="H198" s="9" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I198" s="9" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F198" s="8" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G198" s="8" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H198" s="8" t="inlineStr">
+        <is>
+          <t>58/73</t>
+        </is>
+      </c>
+      <c r="I198" s="8" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -11416,45 +11420,49 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B243" s="9" t="inlineStr">
+      <c r="A243" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B243" s="8" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C243" s="9" t="inlineStr">
+      <c r="C243" s="8" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D243" s="9" t="inlineStr">
+      <c r="D243" s="8" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E243" s="9" t="inlineStr">
+      <c r="E243" s="8" t="inlineStr">
         <is>
           <t>15/06/2026</t>
         </is>
       </c>
-      <c r="F243" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G243" s="9" t="inlineStr"/>
-      <c r="H243" s="9" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I243" s="9" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F243" s="8" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G243" s="8" t="inlineStr">
+        <is>
+          <t>2027/2028</t>
+        </is>
+      </c>
+      <c r="H243" s="8" t="inlineStr">
+        <is>
+          <t>27/37</t>
+        </is>
+      </c>
+      <c r="I243" s="8" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-16 06:18:24 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9">
@@ -1289,10 +1289,10 @@
         <v>14</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
@@ -1367,10 +1367,10 @@
         <v>8</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
@@ -1445,10 +1445,10 @@
         <v>1</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
@@ -1523,10 +1523,10 @@
         <v>6</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q18" s="4" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
@@ -1601,10 +1601,10 @@
         <v>14</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
@@ -2313,45 +2313,45 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E34" s="9" t="inlineStr">
         <is>
           <t>16/06/2026</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr"/>
+      <c r="H34" s="9" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I34" s="9" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -3459,45 +3459,45 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B60" s="9" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C60" s="9" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D60" s="9" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E60" s="9" t="inlineStr">
         <is>
           <t>16/06/2026</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G60" s="2" t="inlineStr"/>
-      <c r="H60" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I60" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F60" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G60" s="9" t="inlineStr"/>
+      <c r="H60" s="9" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I60" s="9" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -6032,45 +6032,45 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B119" s="2" t="inlineStr">
+      <c r="A119" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B119" s="9" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C119" s="2" t="inlineStr">
+      <c r="C119" s="9" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D119" s="2" t="inlineStr">
+      <c r="D119" s="9" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E119" s="2" t="inlineStr">
+      <c r="E119" s="9" t="inlineStr">
         <is>
           <t>16/06/2026</t>
         </is>
       </c>
-      <c r="F119" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G119" s="2" t="inlineStr"/>
-      <c r="H119" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I119" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F119" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G119" s="9" t="inlineStr"/>
+      <c r="H119" s="9" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I119" s="9" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -9496,45 +9496,45 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B199" s="2" t="inlineStr">
+      <c r="A199" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B199" s="9" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C199" s="2" t="inlineStr">
+      <c r="C199" s="9" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D199" s="2" t="inlineStr">
+      <c r="D199" s="9" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E199" s="2" t="inlineStr">
+      <c r="E199" s="9" t="inlineStr">
         <is>
           <t>16/06/2026</t>
         </is>
       </c>
-      <c r="F199" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G199" s="2" t="inlineStr"/>
-      <c r="H199" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I199" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F199" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G199" s="9" t="inlineStr"/>
+      <c r="H199" s="9" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I199" s="9" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -11471,45 +11471,45 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B244" s="2" t="inlineStr">
+      <c r="A244" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B244" s="9" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C244" s="2" t="inlineStr">
+      <c r="C244" s="9" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D244" s="2" t="inlineStr">
+      <c r="D244" s="9" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E244" s="2" t="inlineStr">
+      <c r="E244" s="9" t="inlineStr">
         <is>
           <t>16/06/2026</t>
         </is>
       </c>
-      <c r="F244" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G244" s="2" t="inlineStr"/>
-      <c r="H244" s="2" t="inlineStr">
+      <c r="F244" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G244" s="9" t="inlineStr"/>
+      <c r="H244" s="9" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I244" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I244" s="9" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-16 11:53:57 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>18.0%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>65.2%</t>
+          <t>64.0%</t>
         </is>
       </c>
     </row>
@@ -1520,22 +1520,22 @@
         <v>50</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>32</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>14.0%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>51.6%</t>
+          <t>47.4%</t>
         </is>
       </c>
     </row>
@@ -1598,22 +1598,22 @@
         <v>50</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>32</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>28.0%</t>
+          <t>30.0%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>67.4%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
@@ -9496,45 +9496,49 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B199" s="9" t="inlineStr">
+      <c r="A199" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B199" s="8" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C199" s="9" t="inlineStr">
+      <c r="C199" s="8" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D199" s="9" t="inlineStr">
+      <c r="D199" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E199" s="9" t="inlineStr">
+      <c r="E199" s="8" t="inlineStr">
         <is>
           <t>16/06/2026</t>
         </is>
       </c>
-      <c r="F199" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G199" s="9" t="inlineStr"/>
-      <c r="H199" s="9" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I199" s="9" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F199" s="8" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G199" s="8" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H199" s="8" t="inlineStr">
+        <is>
+          <t>16/73</t>
+        </is>
+      </c>
+      <c r="I199" s="8" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -11471,45 +11475,49 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B244" s="9" t="inlineStr">
+      <c r="A244" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B244" s="8" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C244" s="9" t="inlineStr">
+      <c r="C244" s="8" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D244" s="9" t="inlineStr">
+      <c r="D244" s="8" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E244" s="9" t="inlineStr">
+      <c r="E244" s="8" t="inlineStr">
         <is>
           <t>16/06/2026</t>
         </is>
       </c>
-      <c r="F244" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G244" s="9" t="inlineStr"/>
-      <c r="H244" s="9" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I244" s="9" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F244" s="8" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G244" s="8" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H244" s="8" t="inlineStr">
+        <is>
+          <t>21/37</t>
+        </is>
+      </c>
+      <c r="I244" s="8" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-16 16:55:19 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>18.4%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>64.0%</t>
+          <t>63.7%</t>
         </is>
       </c>
     </row>
@@ -1286,22 +1286,22 @@
         <v>50</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>32</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>28.0%</t>
+          <t>30.0%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>70.5%</t>
+          <t>68.9%</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>47.4%</t>
+          <t>47.7%</t>
         </is>
       </c>
     </row>
@@ -2313,45 +2313,49 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="D34" s="8" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E34" s="9" t="inlineStr">
+      <c r="E34" s="8" t="inlineStr">
         <is>
           <t>16/06/2026</t>
         </is>
       </c>
-      <c r="F34" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G34" s="9" t="inlineStr"/>
-      <c r="H34" s="9" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I34" s="9" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>34/73</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -9533,7 +9537,7 @@
       </c>
       <c r="H199" s="8" t="inlineStr">
         <is>
-          <t>16/73</t>
+          <t>18/73</t>
         </is>
       </c>
       <c r="I199" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-17 13:13:27 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>18.4%</t>
+          <t>19.6%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>63.7%</t>
+          <t>62.0%</t>
         </is>
       </c>
     </row>
@@ -1286,22 +1286,22 @@
         <v>50</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>31</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>30.0%</t>
+          <t>32.0%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>68.9%</t>
+          <t>66.3%</t>
         </is>
       </c>
     </row>
@@ -1520,22 +1520,22 @@
         <v>50</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>31</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>14.0%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>47.7%</t>
+          <t>49.3%</t>
         </is>
       </c>
     </row>
@@ -1598,22 +1598,22 @@
         <v>50</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>31</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>30.0%</t>
+          <t>32.0%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>63.9%</t>
         </is>
       </c>
     </row>
@@ -2360,45 +2360,49 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D35" s="8" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E35" s="9" t="inlineStr">
+      <c r="E35" s="8" t="inlineStr">
         <is>
           <t>17/06/2026</t>
         </is>
       </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G35" s="9" t="inlineStr"/>
-      <c r="H35" s="9" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I35" s="9" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>19/73</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -9547,45 +9551,49 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B200" s="9" t="inlineStr">
+      <c r="A200" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B200" s="8" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C200" s="9" t="inlineStr">
+      <c r="C200" s="8" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D200" s="9" t="inlineStr">
+      <c r="D200" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E200" s="9" t="inlineStr">
+      <c r="E200" s="8" t="inlineStr">
         <is>
           <t>17/06/2026</t>
         </is>
       </c>
-      <c r="F200" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G200" s="9" t="inlineStr"/>
-      <c r="H200" s="9" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I200" s="9" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F200" s="8" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G200" s="8" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H200" s="8" t="inlineStr">
+        <is>
+          <t>44/73</t>
+        </is>
+      </c>
+      <c r="I200" s="8" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -11526,45 +11534,49 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B245" s="9" t="inlineStr">
+      <c r="A245" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B245" s="8" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C245" s="9" t="inlineStr">
+      <c r="C245" s="8" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D245" s="9" t="inlineStr">
+      <c r="D245" s="8" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E245" s="9" t="inlineStr">
+      <c r="E245" s="8" t="inlineStr">
         <is>
           <t>17/06/2026</t>
         </is>
       </c>
-      <c r="F245" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G245" s="9" t="inlineStr"/>
-      <c r="H245" s="9" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I245" s="9" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F245" s="8" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G245" s="8" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H245" s="8" t="inlineStr">
+        <is>
+          <t>8/37</t>
+        </is>
+      </c>
+      <c r="I245" s="8" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-21 08:39:53 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -592,45 +592,45 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>21/06/2026</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
       <c r="K3" s="1" t="inlineStr">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="5" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="L8" s="5" t="n">
-        <v>149</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9">
@@ -1289,10 +1289,10 @@
         <v>16</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q15" s="5" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="R15" s="5" t="inlineStr">
         <is>
@@ -1367,10 +1367,10 @@
         <v>8</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q16" s="5" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="R16" s="5" t="inlineStr">
         <is>
@@ -1445,10 +1445,10 @@
         <v>1</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q17" s="5" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="R17" s="5" t="inlineStr">
         <is>
@@ -1523,10 +1523,10 @@
         <v>8</v>
       </c>
       <c r="P18" s="5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q18" s="5" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="R18" s="5" t="inlineStr">
         <is>
@@ -1601,10 +1601,10 @@
         <v>18</v>
       </c>
       <c r="P19" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q19" s="5" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="R19" s="5" t="inlineStr">
         <is>
@@ -3553,45 +3553,45 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="4" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B62" s="4" t="inlineStr">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D62" s="4" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E62" s="4" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>21/06/2026</t>
         </is>
       </c>
-      <c r="F62" s="4" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G62" s="4" t="inlineStr"/>
-      <c r="H62" s="4" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I62" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -6169,45 +6169,45 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="4" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B122" s="4" t="inlineStr">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C122" s="4" t="inlineStr">
+      <c r="C122" s="2" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D122" s="4" t="inlineStr">
+      <c r="D122" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E122" s="4" t="inlineStr">
+      <c r="E122" s="2" t="inlineStr">
         <is>
           <t>21/06/2026</t>
         </is>
       </c>
-      <c r="F122" s="4" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G122" s="4" t="inlineStr"/>
-      <c r="H122" s="4" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I122" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr"/>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I122" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -8980,45 +8980,45 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="4" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B187" s="4" t="inlineStr">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C187" s="4" t="inlineStr">
+      <c r="C187" s="2" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D187" s="4" t="inlineStr">
+      <c r="D187" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E187" s="4" t="inlineStr">
+      <c r="E187" s="2" t="inlineStr">
         <is>
           <t>21/06/2026</t>
         </is>
       </c>
-      <c r="F187" s="4" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G187" s="4" t="inlineStr"/>
-      <c r="H187" s="4" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I187" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F187" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G187" s="2" t="inlineStr"/>
+      <c r="H187" s="2" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I187" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -10736,45 +10736,45 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="4" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B227" s="4" t="inlineStr">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B227" s="2" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C227" s="4" t="inlineStr">
+      <c r="C227" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D227" s="4" t="inlineStr">
+      <c r="D227" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E227" s="4" t="inlineStr">
+      <c r="E227" s="2" t="inlineStr">
         <is>
           <t>21/06/2026</t>
         </is>
       </c>
-      <c r="F227" s="4" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G227" s="4" t="inlineStr"/>
-      <c r="H227" s="4" t="inlineStr">
+      <c r="F227" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G227" s="2" t="inlineStr"/>
+      <c r="H227" s="2" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I227" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I227" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-21 11:44:26 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="5" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="5" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>20.4%</t>
+          <t>20.8%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>61.0%</t>
+          <t>60.6%</t>
         </is>
       </c>
     </row>
@@ -1598,22 +1598,22 @@
         <v>50</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P19" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q19" s="5" t="n">
         <v>29</v>
       </c>
       <c r="R19" s="5" t="inlineStr">
         <is>
-          <t>36.0%</t>
+          <t>38.0%</t>
         </is>
       </c>
       <c r="S19" s="5" t="inlineStr">
         <is>
-          <t>60.8%</t>
+          <t>59.7%</t>
         </is>
       </c>
     </row>
@@ -10736,45 +10736,49 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B227" s="2" t="inlineStr">
+      <c r="A227" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B227" s="9" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C227" s="2" t="inlineStr">
+      <c r="C227" s="9" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D227" s="2" t="inlineStr">
+      <c r="D227" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E227" s="2" t="inlineStr">
+      <c r="E227" s="9" t="inlineStr">
         <is>
           <t>21/06/2026</t>
         </is>
       </c>
-      <c r="F227" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G227" s="2" t="inlineStr"/>
-      <c r="H227" s="2" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I227" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F227" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G227" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H227" s="9" t="inlineStr">
+        <is>
+          <t>15/37</t>
+        </is>
+      </c>
+      <c r="I227" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-22 13:45:45 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>20.8%</t>
+          <t>21.6%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>60.6%</t>
+          <t>61.2%</t>
         </is>
       </c>
     </row>
@@ -1520,22 +1520,22 @@
         <v>50</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>28</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>18.0%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>49.3%</t>
+          <t>54.3%</t>
         </is>
       </c>
     </row>
@@ -1598,17 +1598,17 @@
         <v>50</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>28</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>38.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
@@ -9023,45 +9023,49 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B188" s="2" t="inlineStr">
+      <c r="A188" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B188" s="9" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C188" s="2" t="inlineStr">
+      <c r="C188" s="9" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D188" s="2" t="inlineStr">
+      <c r="D188" s="9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E188" s="2" t="inlineStr">
+      <c r="E188" s="9" t="inlineStr">
         <is>
           <t>22/06/2026</t>
         </is>
       </c>
-      <c r="F188" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G188" s="2" t="inlineStr"/>
-      <c r="H188" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I188" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F188" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G188" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H188" s="9" t="inlineStr">
+        <is>
+          <t>69/73</t>
+        </is>
+      </c>
+      <c r="I188" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -10783,45 +10787,49 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B228" s="2" t="inlineStr">
+      <c r="A228" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B228" s="9" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C228" s="2" t="inlineStr">
+      <c r="C228" s="9" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D228" s="2" t="inlineStr">
+      <c r="D228" s="9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E228" s="2" t="inlineStr">
+      <c r="E228" s="9" t="inlineStr">
         <is>
           <t>22/06/2026</t>
         </is>
       </c>
-      <c r="F228" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G228" s="2" t="inlineStr"/>
-      <c r="H228" s="2" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I228" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F228" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G228" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H228" s="9" t="inlineStr">
+        <is>
+          <t>22/37</t>
+        </is>
+      </c>
+      <c r="I228" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-24 10:34:10 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>22.4%</t>
+          <t>22.8%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>60.3%</t>
+          <t>60.0%</t>
         </is>
       </c>
     </row>
@@ -1598,22 +1598,22 @@
         <v>50</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>26</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>42.0%</t>
+          <t>44.0%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>59.3%</t>
+          <t>58.6%</t>
         </is>
       </c>
     </row>
@@ -10885,45 +10885,49 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B230" s="2" t="inlineStr">
+      <c r="A230" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B230" s="9" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C230" s="2" t="inlineStr">
+      <c r="C230" s="9" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D230" s="2" t="inlineStr">
+      <c r="D230" s="9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E230" s="2" t="inlineStr">
+      <c r="E230" s="9" t="inlineStr">
         <is>
           <t>24/06/2026</t>
         </is>
       </c>
-      <c r="F230" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G230" s="2" t="inlineStr"/>
-      <c r="H230" s="2" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I230" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F230" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G230" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H230" s="9" t="inlineStr">
+        <is>
+          <t>16/37</t>
+        </is>
+      </c>
+      <c r="I230" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-24 12:47:16 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>22.8%</t>
+          <t>23.2%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>62.5%</t>
         </is>
       </c>
     </row>
@@ -1520,22 +1520,22 @@
         <v>50</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>26</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>22.0%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>50.8%</t>
+          <t>59.8%</t>
         </is>
       </c>
     </row>
@@ -1613,7 +1613,7 @@
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>58.6%</t>
+          <t>61.2%</t>
         </is>
       </c>
     </row>
@@ -9102,12 +9102,12 @@
       </c>
       <c r="G189" s="9" t="inlineStr">
         <is>
-          <t>2026/2027</t>
+          <t>2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H189" s="9" t="inlineStr">
         <is>
-          <t>14/73</t>
+          <t>63/73</t>
         </is>
       </c>
       <c r="I189" s="9" t="inlineStr">
@@ -9117,45 +9117,49 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B190" s="2" t="inlineStr">
+      <c r="A190" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B190" s="9" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C190" s="2" t="inlineStr">
+      <c r="C190" s="9" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D190" s="2" t="inlineStr">
+      <c r="D190" s="9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E190" s="2" t="inlineStr">
+      <c r="E190" s="9" t="inlineStr">
         <is>
           <t>24/06/2026</t>
         </is>
       </c>
-      <c r="F190" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G190" s="2" t="inlineStr"/>
-      <c r="H190" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I190" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F190" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G190" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H190" s="9" t="inlineStr">
+        <is>
+          <t>60/73</t>
+        </is>
+      </c>
+      <c r="I190" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -11368,7 +11372,7 @@
       </c>
       <c r="H240" s="9" t="inlineStr">
         <is>
-          <t>5/37</t>
+          <t>26/37</t>
         </is>
       </c>
       <c r="I240" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-25 08:34:14 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9">
@@ -1367,10 +1367,10 @@
         <v>8</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
@@ -1445,10 +1445,10 @@
         <v>1</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
@@ -1523,10 +1523,10 @@
         <v>11</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q18" s="4" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
@@ -1601,10 +1601,10 @@
         <v>22</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
@@ -3725,45 +3725,45 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B66" s="5" t="inlineStr">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C66" s="5" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D66" s="5" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E66" s="5" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>25/06/2026</t>
         </is>
       </c>
-      <c r="F66" s="5" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G66" s="5" t="inlineStr"/>
-      <c r="H66" s="5" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I66" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr"/>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -6341,45 +6341,45 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B126" s="5" t="inlineStr">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C126" s="5" t="inlineStr">
+      <c r="C126" s="2" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D126" s="5" t="inlineStr">
+      <c r="D126" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E126" s="5" t="inlineStr">
+      <c r="E126" s="2" t="inlineStr">
         <is>
           <t>25/06/2026</t>
         </is>
       </c>
-      <c r="F126" s="5" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G126" s="5" t="inlineStr"/>
-      <c r="H126" s="5" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I126" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr"/>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I126" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -9164,45 +9164,45 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B191" s="5" t="inlineStr">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C191" s="5" t="inlineStr">
+      <c r="C191" s="2" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D191" s="5" t="inlineStr">
+      <c r="D191" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E191" s="5" t="inlineStr">
+      <c r="E191" s="2" t="inlineStr">
         <is>
           <t>25/06/2026</t>
         </is>
       </c>
-      <c r="F191" s="5" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G191" s="5" t="inlineStr"/>
-      <c r="H191" s="5" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I191" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F191" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G191" s="2" t="inlineStr"/>
+      <c r="H191" s="2" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I191" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -10936,45 +10936,45 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B231" s="5" t="inlineStr">
+      <c r="A231" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B231" s="2" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C231" s="5" t="inlineStr">
+      <c r="C231" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D231" s="5" t="inlineStr">
+      <c r="D231" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E231" s="5" t="inlineStr">
+      <c r="E231" s="2" t="inlineStr">
         <is>
           <t>25/06/2026</t>
         </is>
       </c>
-      <c r="F231" s="5" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G231" s="5" t="inlineStr"/>
-      <c r="H231" s="5" t="inlineStr">
+      <c r="F231" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G231" s="2" t="inlineStr"/>
+      <c r="H231" s="2" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I231" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I231" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-25 11:28:36 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>23.2%</t>
+          <t>23.6%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>62.5%</t>
+          <t>62.2%</t>
         </is>
       </c>
     </row>
@@ -1598,22 +1598,22 @@
         <v>50</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>25</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>44.0%</t>
+          <t>46.0%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>61.2%</t>
+          <t>60.4%</t>
         </is>
       </c>
     </row>
@@ -10936,45 +10936,49 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B231" s="2" t="inlineStr">
+      <c r="A231" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B231" s="9" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C231" s="2" t="inlineStr">
+      <c r="C231" s="9" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D231" s="2" t="inlineStr">
+      <c r="D231" s="9" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E231" s="2" t="inlineStr">
+      <c r="E231" s="9" t="inlineStr">
         <is>
           <t>25/06/2026</t>
         </is>
       </c>
-      <c r="F231" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G231" s="2" t="inlineStr"/>
-      <c r="H231" s="2" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I231" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F231" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G231" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H231" s="9" t="inlineStr">
+        <is>
+          <t>16/37</t>
+        </is>
+      </c>
+      <c r="I231" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-30 11:40:56 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>26.0%</t>
+          <t>27.2%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>62.2%</t>
+          <t>61.6%</t>
         </is>
       </c>
     </row>
@@ -1442,22 +1442,22 @@
         <v>50</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>22</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>8.0%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>84.9%</t>
+          <t>82.5%</t>
         </is>
       </c>
     </row>
@@ -1520,22 +1520,22 @@
         <v>50</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>22</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>26.0%</t>
+          <t>28.0%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>63.8%</t>
+          <t>63.9%</t>
         </is>
       </c>
     </row>
@@ -1598,22 +1598,22 @@
         <v>50</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>22</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>52.0%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>57.4%</t>
+          <t>55.4%</t>
         </is>
       </c>
     </row>
@@ -7338,45 +7338,49 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B149" s="2" t="inlineStr">
+      <c r="A149" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B149" s="9" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C149" s="2" t="inlineStr">
+      <c r="C149" s="9" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D149" s="2" t="inlineStr">
+      <c r="D149" s="9" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E149" s="2" t="inlineStr">
+      <c r="E149" s="9" t="inlineStr">
         <is>
           <t>30/06/2026</t>
         </is>
       </c>
-      <c r="F149" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G149" s="2" t="inlineStr"/>
-      <c r="H149" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I149" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F149" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G149" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H149" s="9" t="inlineStr">
+        <is>
+          <t>55/73</t>
+        </is>
+      </c>
+      <c r="I149" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -9309,45 +9313,49 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B194" s="2" t="inlineStr">
+      <c r="A194" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B194" s="9" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C194" s="2" t="inlineStr">
+      <c r="C194" s="9" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D194" s="2" t="inlineStr">
+      <c r="D194" s="9" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E194" s="2" t="inlineStr">
+      <c r="E194" s="9" t="inlineStr">
         <is>
           <t>30/06/2026</t>
         </is>
       </c>
-      <c r="F194" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G194" s="2" t="inlineStr"/>
-      <c r="H194" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I194" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F194" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G194" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H194" s="9" t="inlineStr">
+        <is>
+          <t>48/73</t>
+        </is>
+      </c>
+      <c r="I194" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -11093,45 +11101,49 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B234" s="2" t="inlineStr">
+      <c r="A234" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B234" s="9" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C234" s="2" t="inlineStr">
+      <c r="C234" s="9" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D234" s="2" t="inlineStr">
+      <c r="D234" s="9" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E234" s="2" t="inlineStr">
+      <c r="E234" s="9" t="inlineStr">
         <is>
           <t>30/06/2026</t>
         </is>
       </c>
-      <c r="F234" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G234" s="2" t="inlineStr"/>
-      <c r="H234" s="2" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I234" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F234" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G234" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H234" s="9" t="inlineStr">
+        <is>
+          <t>2/37</t>
+        </is>
+      </c>
+      <c r="I234" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-30 18:33:23 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>61.6%</t>
+          <t>61.7%</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>82.5%</t>
+          <t>83.6%</t>
         </is>
       </c>
     </row>
@@ -7375,7 +7375,7 @@
       </c>
       <c r="H149" s="9" t="inlineStr">
         <is>
-          <t>55/73</t>
+          <t>58/73</t>
         </is>
       </c>
       <c r="I149" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-01 13:32:41 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>27.2%</t>
+          <t>28.4%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>61.7%</t>
+          <t>60.4%</t>
         </is>
       </c>
     </row>
@@ -1442,22 +1442,22 @@
         <v>50</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>21</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>8.0%</t>
+          <t>10.0%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>83.6%</t>
+          <t>67.1%</t>
         </is>
       </c>
     </row>
@@ -1520,22 +1520,22 @@
         <v>50</v>
       </c>
       <c r="O18" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="P18" s="4" t="n">
         <v>14</v>
-      </c>
-      <c r="P18" s="4" t="n">
-        <v>15</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>21</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>28.0%</t>
+          <t>30.0%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>63.9%</t>
+          <t>64.7%</t>
         </is>
       </c>
     </row>
@@ -1598,22 +1598,22 @@
         <v>50</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>21</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>52.0%</t>
+          <t>54.0%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>55.4%</t>
+          <t>54.2%</t>
         </is>
       </c>
     </row>
@@ -7385,45 +7385,49 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B150" s="2" t="inlineStr">
+      <c r="A150" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B150" s="9" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C150" s="2" t="inlineStr">
+      <c r="C150" s="9" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D150" s="2" t="inlineStr">
+      <c r="D150" s="9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E150" s="2" t="inlineStr">
+      <c r="E150" s="9" t="inlineStr">
         <is>
           <t>01/07/2026</t>
         </is>
       </c>
-      <c r="F150" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G150" s="2" t="inlineStr"/>
-      <c r="H150" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I150" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F150" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G150" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H150" s="9" t="inlineStr">
+        <is>
+          <t>1/73</t>
+        </is>
+      </c>
+      <c r="I150" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -9360,45 +9364,49 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B195" s="2" t="inlineStr">
+      <c r="A195" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B195" s="9" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C195" s="2" t="inlineStr">
+      <c r="C195" s="9" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D195" s="2" t="inlineStr">
+      <c r="D195" s="9" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E195" s="2" t="inlineStr">
+      <c r="E195" s="9" t="inlineStr">
         <is>
           <t>01/07/2026</t>
         </is>
       </c>
-      <c r="F195" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G195" s="2" t="inlineStr"/>
-      <c r="H195" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I195" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F195" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G195" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H195" s="9" t="inlineStr">
+        <is>
+          <t>55/73</t>
+        </is>
+      </c>
+      <c r="I195" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -11148,45 +11156,49 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B235" s="2" t="inlineStr">
+      <c r="A235" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B235" s="9" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C235" s="2" t="inlineStr">
+      <c r="C235" s="9" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D235" s="2" t="inlineStr">
+      <c r="D235" s="9" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E235" s="2" t="inlineStr">
+      <c r="E235" s="9" t="inlineStr">
         <is>
           <t>01/07/2026</t>
         </is>
       </c>
-      <c r="F235" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G235" s="2" t="inlineStr"/>
-      <c r="H235" s="2" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I235" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F235" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G235" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H235" s="9" t="inlineStr">
+        <is>
+          <t>8/37</t>
+        </is>
+      </c>
+      <c r="I235" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-04 20:19:06 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9">
@@ -1367,10 +1367,10 @@
         <v>8</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
@@ -1445,10 +1445,10 @@
         <v>5</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
@@ -1523,10 +1523,10 @@
         <v>15</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q18" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
@@ -1601,10 +1601,10 @@
         <v>27</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
@@ -3940,45 +3940,45 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B71" s="5" t="inlineStr">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C71" s="5" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D71" s="5" t="inlineStr">
+      <c r="D71" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E71" s="5" t="inlineStr">
+      <c r="E71" s="2" t="inlineStr">
         <is>
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F71" s="5" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G71" s="5" t="inlineStr"/>
-      <c r="H71" s="5" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I71" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr"/>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -7432,45 +7432,45 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B151" s="5" t="inlineStr">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C151" s="5" t="inlineStr">
+      <c r="C151" s="2" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D151" s="5" t="inlineStr">
+      <c r="D151" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E151" s="5" t="inlineStr">
+      <c r="E151" s="2" t="inlineStr">
         <is>
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F151" s="5" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G151" s="5" t="inlineStr"/>
-      <c r="H151" s="5" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I151" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr"/>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I151" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -9411,45 +9411,45 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B196" s="5" t="inlineStr">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C196" s="5" t="inlineStr">
+      <c r="C196" s="2" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D196" s="5" t="inlineStr">
+      <c r="D196" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E196" s="5" t="inlineStr">
+      <c r="E196" s="2" t="inlineStr">
         <is>
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F196" s="5" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G196" s="5" t="inlineStr"/>
-      <c r="H196" s="5" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I196" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F196" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G196" s="2" t="inlineStr"/>
+      <c r="H196" s="2" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I196" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -9685,45 +9685,45 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B202" s="5" t="inlineStr">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C202" s="5" t="inlineStr">
+      <c r="C202" s="2" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D202" s="5" t="inlineStr">
+      <c r="D202" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E202" s="5" t="inlineStr">
+      <c r="E202" s="2" t="inlineStr">
         <is>
           <t>04/07/2026</t>
         </is>
       </c>
-      <c r="F202" s="5" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G202" s="5" t="inlineStr"/>
-      <c r="H202" s="5" t="inlineStr">
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr"/>
+      <c r="H202" s="2" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I202" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I202" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -11203,45 +11203,45 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B236" s="5" t="inlineStr">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C236" s="5" t="inlineStr">
+      <c r="C236" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D236" s="5" t="inlineStr">
+      <c r="D236" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E236" s="5" t="inlineStr">
+      <c r="E236" s="2" t="inlineStr">
         <is>
           <t>02/07/2026</t>
         </is>
       </c>
-      <c r="F236" s="5" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G236" s="5" t="inlineStr"/>
-      <c r="H236" s="5" t="inlineStr">
+      <c r="F236" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G236" s="2" t="inlineStr"/>
+      <c r="H236" s="2" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I236" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I236" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-04 21:06:37 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>71</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>28.4%</t>
+          <t>32.4%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>61.4%</t>
+          <t>64.8%</t>
         </is>
       </c>
     </row>
@@ -1442,22 +1442,22 @@
         <v>50</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>20</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>80.8%</t>
+          <t>86.3%</t>
         </is>
       </c>
     </row>
@@ -1520,22 +1520,22 @@
         <v>50</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>20</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>30.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>64.7%</t>
+          <t>70.0%</t>
         </is>
       </c>
     </row>
@@ -6169,217 +6169,237 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B122" s="2" t="inlineStr">
+      <c r="A122" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B122" s="9" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C122" s="2" t="inlineStr">
+      <c r="C122" s="9" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D122" s="2" t="inlineStr">
+      <c r="D122" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E122" s="2" t="inlineStr">
+      <c r="E122" s="9" t="inlineStr">
         <is>
           <t>21/06/2026</t>
         </is>
       </c>
-      <c r="F122" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G122" s="2" t="inlineStr"/>
-      <c r="H122" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I122" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F122" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G122" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H122" s="9" t="inlineStr">
+        <is>
+          <t>66/73</t>
+        </is>
+      </c>
+      <c r="I122" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B123" s="2" t="inlineStr">
+      <c r="A123" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B123" s="9" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C123" s="2" t="inlineStr">
+      <c r="C123" s="9" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D123" s="2" t="inlineStr">
+      <c r="D123" s="9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E123" s="2" t="inlineStr">
+      <c r="E123" s="9" t="inlineStr">
         <is>
           <t>22/06/2026</t>
         </is>
       </c>
-      <c r="F123" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G123" s="2" t="inlineStr"/>
-      <c r="H123" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I123" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F123" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G123" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H123" s="9" t="inlineStr">
+        <is>
+          <t>59/73</t>
+        </is>
+      </c>
+      <c r="I123" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B124" s="2" t="inlineStr">
+      <c r="A124" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B124" s="9" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C124" s="2" t="inlineStr">
+      <c r="C124" s="9" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D124" s="2" t="inlineStr">
+      <c r="D124" s="9" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E124" s="2" t="inlineStr">
+      <c r="E124" s="9" t="inlineStr">
         <is>
           <t>23/06/2026</t>
         </is>
       </c>
-      <c r="F124" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G124" s="2" t="inlineStr"/>
-      <c r="H124" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I124" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F124" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G124" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H124" s="9" t="inlineStr">
+        <is>
+          <t>72/73</t>
+        </is>
+      </c>
+      <c r="I124" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B125" s="2" t="inlineStr">
+      <c r="A125" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B125" s="9" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C125" s="2" t="inlineStr">
+      <c r="C125" s="9" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D125" s="2" t="inlineStr">
+      <c r="D125" s="9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E125" s="2" t="inlineStr">
+      <c r="E125" s="9" t="inlineStr">
         <is>
           <t>24/06/2026</t>
         </is>
       </c>
-      <c r="F125" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G125" s="2" t="inlineStr"/>
-      <c r="H125" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I125" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F125" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G125" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H125" s="9" t="inlineStr">
+        <is>
+          <t>67/73</t>
+        </is>
+      </c>
+      <c r="I125" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B126" s="2" t="inlineStr">
+      <c r="A126" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B126" s="9" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C126" s="2" t="inlineStr">
+      <c r="C126" s="9" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D126" s="2" t="inlineStr">
+      <c r="D126" s="9" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E126" s="2" t="inlineStr">
+      <c r="E126" s="9" t="inlineStr">
         <is>
           <t>25/06/2026</t>
         </is>
       </c>
-      <c r="F126" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G126" s="2" t="inlineStr"/>
-      <c r="H126" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I126" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F126" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G126" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H126" s="9" t="inlineStr">
+        <is>
+          <t>71/73</t>
+        </is>
+      </c>
+      <c r="I126" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -8351,217 +8371,237 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B172" s="2" t="inlineStr">
+      <c r="A172" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B172" s="9" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C172" s="2" t="inlineStr">
+      <c r="C172" s="9" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D172" s="2" t="inlineStr">
+      <c r="D172" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E172" s="2" t="inlineStr">
+      <c r="E172" s="9" t="inlineStr">
         <is>
           <t>07/06/2026</t>
         </is>
       </c>
-      <c r="F172" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G172" s="2" t="inlineStr"/>
-      <c r="H172" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I172" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F172" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G172" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H172" s="9" t="inlineStr">
+        <is>
+          <t>67/73</t>
+        </is>
+      </c>
+      <c r="I172" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B173" s="2" t="inlineStr">
+      <c r="A173" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B173" s="9" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C173" s="2" t="inlineStr">
+      <c r="C173" s="9" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D173" s="2" t="inlineStr">
+      <c r="D173" s="9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E173" s="2" t="inlineStr">
+      <c r="E173" s="9" t="inlineStr">
         <is>
           <t>08/06/2026</t>
         </is>
       </c>
-      <c r="F173" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G173" s="2" t="inlineStr"/>
-      <c r="H173" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I173" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F173" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G173" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H173" s="9" t="inlineStr">
+        <is>
+          <t>65/73</t>
+        </is>
+      </c>
+      <c r="I173" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B174" s="2" t="inlineStr">
+      <c r="A174" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B174" s="9" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C174" s="2" t="inlineStr">
+      <c r="C174" s="9" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D174" s="2" t="inlineStr">
+      <c r="D174" s="9" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E174" s="2" t="inlineStr">
+      <c r="E174" s="9" t="inlineStr">
         <is>
           <t>09/06/2026</t>
         </is>
       </c>
-      <c r="F174" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G174" s="2" t="inlineStr"/>
-      <c r="H174" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I174" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F174" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G174" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H174" s="9" t="inlineStr">
+        <is>
+          <t>69/73</t>
+        </is>
+      </c>
+      <c r="I174" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B175" s="2" t="inlineStr">
+      <c r="A175" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B175" s="9" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C175" s="2" t="inlineStr">
+      <c r="C175" s="9" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D175" s="2" t="inlineStr">
+      <c r="D175" s="9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E175" s="2" t="inlineStr">
+      <c r="E175" s="9" t="inlineStr">
         <is>
           <t>10/06/2026</t>
         </is>
       </c>
-      <c r="F175" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G175" s="2" t="inlineStr"/>
-      <c r="H175" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I175" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F175" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G175" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H175" s="9" t="inlineStr">
+        <is>
+          <t>61/73</t>
+        </is>
+      </c>
+      <c r="I175" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B176" s="2" t="inlineStr">
+      <c r="A176" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B176" s="9" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C176" s="2" t="inlineStr">
+      <c r="C176" s="9" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D176" s="2" t="inlineStr">
+      <c r="D176" s="9" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E176" s="2" t="inlineStr">
+      <c r="E176" s="9" t="inlineStr">
         <is>
           <t>11/06/2026</t>
         </is>
       </c>
-      <c r="F176" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G176" s="2" t="inlineStr"/>
-      <c r="H176" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I176" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F176" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G176" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H176" s="9" t="inlineStr">
+        <is>
+          <t>52/73</t>
+        </is>
+      </c>
+      <c r="I176" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-07 12:39:04 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>33.6%</t>
+          <t>34.4%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>64.8%</t>
+          <t>64.6%</t>
         </is>
       </c>
     </row>
@@ -1442,22 +1442,22 @@
         <v>50</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>17</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>22.0%</t>
+          <t>24.0%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>87.5%</t>
+          <t>87.8%</t>
         </is>
       </c>
     </row>
@@ -1520,22 +1520,22 @@
         <v>50</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>17</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>44.0%</t>
+          <t>46.0%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>67.8%</t>
+          <t>66.0%</t>
         </is>
       </c>
     </row>
@@ -6924,45 +6924,49 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B139" s="2" t="inlineStr">
+      <c r="A139" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B139" s="9" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C139" s="2" t="inlineStr">
+      <c r="C139" s="9" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D139" s="2" t="inlineStr">
+      <c r="D139" s="9" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E139" s="2" t="inlineStr">
+      <c r="E139" s="9" t="inlineStr">
         <is>
           <t>07/07/2026</t>
         </is>
       </c>
-      <c r="F139" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G139" s="2" t="inlineStr"/>
-      <c r="H139" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I139" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F139" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G139" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H139" s="9" t="inlineStr">
+        <is>
+          <t>66/73</t>
+        </is>
+      </c>
+      <c r="I139" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -8704,45 +8708,49 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B179" s="2" t="inlineStr">
+      <c r="A179" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B179" s="9" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C179" s="2" t="inlineStr">
+      <c r="C179" s="9" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D179" s="2" t="inlineStr">
+      <c r="D179" s="9" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E179" s="2" t="inlineStr">
+      <c r="E179" s="9" t="inlineStr">
         <is>
           <t>07/07/2026</t>
         </is>
       </c>
-      <c r="F179" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G179" s="2" t="inlineStr"/>
-      <c r="H179" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I179" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F179" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G179" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H179" s="9" t="inlineStr">
+        <is>
+          <t>19/73</t>
+        </is>
+      </c>
+      <c r="I179" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-08 12:31:15 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>34.8%</t>
+          <t>35.2%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>64.4%</t>
+          <t>64.6%</t>
         </is>
       </c>
     </row>
@@ -1442,22 +1442,22 @@
         <v>50</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>16</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>24.0%</t>
+          <t>26.0%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>87.8%</t>
+          <t>87.5%</t>
         </is>
       </c>
     </row>
@@ -6971,45 +6971,49 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B140" s="2" t="inlineStr">
+      <c r="A140" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B140" s="9" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C140" s="2" t="inlineStr">
+      <c r="C140" s="9" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D140" s="2" t="inlineStr">
+      <c r="D140" s="9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E140" s="2" t="inlineStr">
+      <c r="E140" s="9" t="inlineStr">
         <is>
           <t>08/07/2026</t>
         </is>
       </c>
-      <c r="F140" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G140" s="2" t="inlineStr"/>
-      <c r="H140" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I140" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F140" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G140" s="9" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="H140" s="9" t="inlineStr">
+        <is>
+          <t>61/73</t>
+        </is>
+      </c>
+      <c r="I140" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-09 11:39:02 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>35.2%</t>
+          <t>36.0%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>64.6%</t>
+          <t>64.3%</t>
         </is>
       </c>
     </row>
@@ -1442,22 +1442,22 @@
         <v>50</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>15</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>26.0%</t>
+          <t>28.0%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>87.5%</t>
+          <t>85.7%</t>
         </is>
       </c>
     </row>
@@ -1520,22 +1520,22 @@
         <v>50</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>15</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>48.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>65.0%</t>
+          <t>64.1%</t>
         </is>
       </c>
     </row>
@@ -7018,45 +7018,49 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B141" s="2" t="inlineStr">
+      <c r="A141" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B141" s="9" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C141" s="2" t="inlineStr">
+      <c r="C141" s="9" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D141" s="2" t="inlineStr">
+      <c r="D141" s="9" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E141" s="2" t="inlineStr">
+      <c r="E141" s="9" t="inlineStr">
         <is>
           <t>09/07/2026</t>
         </is>
       </c>
-      <c r="F141" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G141" s="2" t="inlineStr"/>
-      <c r="H141" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I141" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F141" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G141" s="9" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="H141" s="9" t="inlineStr">
+        <is>
+          <t>46/73</t>
+        </is>
+      </c>
+      <c r="I141" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -8806,45 +8810,49 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B181" s="2" t="inlineStr">
+      <c r="A181" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B181" s="9" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C181" s="2" t="inlineStr">
+      <c r="C181" s="9" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D181" s="2" t="inlineStr">
+      <c r="D181" s="9" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E181" s="2" t="inlineStr">
+      <c r="E181" s="9" t="inlineStr">
         <is>
           <t>09/07/2026</t>
         </is>
       </c>
-      <c r="F181" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G181" s="2" t="inlineStr"/>
-      <c r="H181" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I181" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F181" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G181" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H181" s="9" t="inlineStr">
+        <is>
+          <t>30/73</t>
+        </is>
+      </c>
+      <c r="I181" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-12 11:06:44 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>36.0%</t>
+          <t>36.4%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>64.3%</t>
+          <t>64.6%</t>
         </is>
       </c>
     </row>
@@ -1442,22 +1442,22 @@
         <v>50</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>14</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>28.0%</t>
+          <t>30.0%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>85.7%</t>
+          <t>85.8%</t>
         </is>
       </c>
     </row>
@@ -7065,45 +7065,49 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B142" s="2" t="inlineStr">
+      <c r="A142" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B142" s="9" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C142" s="2" t="inlineStr">
+      <c r="C142" s="9" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D142" s="2" t="inlineStr">
+      <c r="D142" s="9" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E142" s="2" t="inlineStr">
+      <c r="E142" s="9" t="inlineStr">
         <is>
           <t>12/07/2026</t>
         </is>
       </c>
-      <c r="F142" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G142" s="2" t="inlineStr"/>
-      <c r="H142" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I142" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F142" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G142" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H142" s="9" t="inlineStr">
+        <is>
+          <t>64/73</t>
+        </is>
+      </c>
+      <c r="I142" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-13 11:49:43 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>36.4%</t>
+          <t>37.6%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>64.6%</t>
+          <t>65.0%</t>
         </is>
       </c>
     </row>
@@ -1364,22 +1364,22 @@
         <v>50</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>13</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>18.0%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>57.9%</t>
+          <t>61.9%</t>
         </is>
       </c>
     </row>
@@ -1442,22 +1442,22 @@
         <v>50</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>13</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>30.0%</t>
+          <t>32.0%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>85.8%</t>
+          <t>86.1%</t>
         </is>
       </c>
     </row>
@@ -1520,22 +1520,22 @@
         <v>50</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>13</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>52.0%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>64.1%</t>
+          <t>63.5%</t>
         </is>
       </c>
     </row>
@@ -5133,45 +5133,49 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B98" s="2" t="inlineStr">
+      <c r="A98" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B98" s="9" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C98" s="2" t="inlineStr">
+      <c r="C98" s="9" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D98" s="2" t="inlineStr">
+      <c r="D98" s="9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E98" s="2" t="inlineStr">
+      <c r="E98" s="9" t="inlineStr">
         <is>
           <t>13/07/2026</t>
         </is>
       </c>
-      <c r="F98" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G98" s="2" t="inlineStr"/>
-      <c r="H98" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I98" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F98" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G98" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H98" s="9" t="inlineStr">
+        <is>
+          <t>69/73</t>
+        </is>
+      </c>
+      <c r="I98" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -7112,45 +7116,49 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B143" s="2" t="inlineStr">
+      <c r="A143" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B143" s="9" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C143" s="2" t="inlineStr">
+      <c r="C143" s="9" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D143" s="2" t="inlineStr">
+      <c r="D143" s="9" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E143" s="2" t="inlineStr">
+      <c r="E143" s="9" t="inlineStr">
         <is>
           <t>13/07/2026</t>
         </is>
       </c>
-      <c r="F143" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G143" s="2" t="inlineStr"/>
-      <c r="H143" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I143" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F143" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G143" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H143" s="9" t="inlineStr">
+        <is>
+          <t>66/73</t>
+        </is>
+      </c>
+      <c r="I143" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -8904,45 +8912,49 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B183" s="2" t="inlineStr">
+      <c r="A183" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B183" s="9" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C183" s="2" t="inlineStr">
+      <c r="C183" s="9" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D183" s="2" t="inlineStr">
+      <c r="D183" s="9" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E183" s="2" t="inlineStr">
+      <c r="E183" s="9" t="inlineStr">
         <is>
           <t>13/07/2026</t>
         </is>
       </c>
-      <c r="F183" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G183" s="2" t="inlineStr"/>
-      <c r="H183" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I183" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F183" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G183" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H183" s="9" t="inlineStr">
+        <is>
+          <t>36/73</t>
+        </is>
+      </c>
+      <c r="I183" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-15 11:23:31 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>38.8%</t>
+          <t>39.6%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>65.3%</t>
+          <t>65.2%</t>
         </is>
       </c>
     </row>
@@ -1442,22 +1442,22 @@
         <v>50</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>11</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>34.0%</t>
+          <t>36.0%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>86.0%</t>
+          <t>85.6%</t>
         </is>
       </c>
     </row>
@@ -1520,22 +1520,22 @@
         <v>50</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>11</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>54.0%</t>
+          <t>56.0%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>63.0%</t>
+          <t>62.4%</t>
         </is>
       </c>
     </row>
@@ -7214,45 +7214,49 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B145" s="2" t="inlineStr">
+      <c r="A145" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B145" s="9" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C145" s="2" t="inlineStr">
+      <c r="C145" s="9" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D145" s="2" t="inlineStr">
+      <c r="D145" s="9" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E145" s="2" t="inlineStr">
+      <c r="E145" s="9" t="inlineStr">
         <is>
           <t>15/07/2026</t>
         </is>
       </c>
-      <c r="F145" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G145" s="2" t="inlineStr"/>
-      <c r="H145" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I145" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F145" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G145" s="9" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="H145" s="9" t="inlineStr">
+        <is>
+          <t>58/73</t>
+        </is>
+      </c>
+      <c r="I145" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -9014,45 +9018,49 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B185" s="2" t="inlineStr">
+      <c r="A185" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B185" s="9" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C185" s="2" t="inlineStr">
+      <c r="C185" s="9" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D185" s="2" t="inlineStr">
+      <c r="D185" s="9" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E185" s="2" t="inlineStr">
+      <c r="E185" s="9" t="inlineStr">
         <is>
           <t>15/07/2026</t>
         </is>
       </c>
-      <c r="F185" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G185" s="2" t="inlineStr"/>
-      <c r="H185" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I185" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F185" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G185" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H185" s="9" t="inlineStr">
+        <is>
+          <t>34/73</t>
+        </is>
+      </c>
+      <c r="I185" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-15 22:18:18 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>39.6%</t>
+          <t>41.2%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>65.2%</t>
+          <t>66.0%</t>
         </is>
       </c>
     </row>
@@ -1364,22 +1364,22 @@
         <v>50</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>11</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>28.0%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>64.8%</t>
+          <t>70.8%</t>
         </is>
       </c>
     </row>
@@ -3983,174 +3983,190 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
+      <c r="A72" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B72" s="9" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr">
+      <c r="C72" s="9" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D72" s="2" t="inlineStr">
+      <c r="D72" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E72" s="2" t="inlineStr">
+      <c r="E72" s="9" t="inlineStr">
         <is>
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F72" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G72" s="2" t="inlineStr"/>
-      <c r="H72" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I72" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F72" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G72" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H72" s="9" t="inlineStr">
+        <is>
+          <t>57/73</t>
+        </is>
+      </c>
+      <c r="I72" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
+      <c r="A73" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B73" s="9" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C73" s="2" t="inlineStr">
+      <c r="C73" s="9" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D73" s="2" t="inlineStr">
+      <c r="D73" s="9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E73" s="2" t="inlineStr">
+      <c r="E73" s="9" t="inlineStr">
         <is>
           <t>06/07/2026</t>
         </is>
       </c>
-      <c r="F73" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G73" s="2" t="inlineStr"/>
-      <c r="H73" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I73" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F73" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G73" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H73" s="9" t="inlineStr">
+        <is>
+          <t>66/73</t>
+        </is>
+      </c>
+      <c r="I73" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
+      <c r="A74" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B74" s="9" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr">
+      <c r="C74" s="9" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D74" s="2" t="inlineStr">
+      <c r="D74" s="9" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E74" s="2" t="inlineStr">
+      <c r="E74" s="9" t="inlineStr">
         <is>
           <t>07/07/2026</t>
         </is>
       </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr"/>
-      <c r="H74" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F74" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G74" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H74" s="9" t="inlineStr">
+        <is>
+          <t>73/73</t>
+        </is>
+      </c>
+      <c r="I74" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B75" s="2" t="inlineStr">
+      <c r="A75" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B75" s="9" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr">
+      <c r="C75" s="9" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D75" s="2" t="inlineStr">
+      <c r="D75" s="9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E75" s="2" t="inlineStr">
+      <c r="E75" s="9" t="inlineStr">
         <is>
           <t>08/07/2026</t>
         </is>
       </c>
-      <c r="F75" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G75" s="2" t="inlineStr"/>
-      <c r="H75" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I75" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F75" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G75" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H75" s="9" t="inlineStr">
+        <is>
+          <t>55/73</t>
+        </is>
+      </c>
+      <c r="I75" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-16 10:16:22 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>41.6%</t>
+          <t>42.0%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>66.3%</t>
+          <t>65.8%</t>
         </is>
       </c>
     </row>
@@ -1520,22 +1520,22 @@
         <v>50</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>10</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>56.0%</t>
+          <t>58.0%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>62.4%</t>
+          <t>60.4%</t>
         </is>
       </c>
     </row>
@@ -9085,45 +9085,49 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B186" s="2" t="inlineStr">
+      <c r="A186" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B186" s="9" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C186" s="2" t="inlineStr">
+      <c r="C186" s="9" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D186" s="2" t="inlineStr">
+      <c r="D186" s="9" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E186" s="2" t="inlineStr">
+      <c r="E186" s="9" t="inlineStr">
         <is>
           <t>16/07/2026</t>
         </is>
       </c>
-      <c r="F186" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G186" s="2" t="inlineStr"/>
-      <c r="H186" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I186" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F186" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G186" s="9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H186" s="9" t="inlineStr">
+        <is>
+          <t>4/73</t>
+        </is>
+      </c>
+      <c r="I186" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-16 16:07:54 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6421,7 +6421,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8612,7 +8612,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8659,7 +8659,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-16 17:25:25 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6421,7 +6421,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8612,7 +8612,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8659,7 +8659,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-16 18:46:23 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6421,7 +6421,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8612,7 +8612,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8659,7 +8659,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-16 20:13:37 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6421,7 +6421,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8612,7 +8612,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8659,7 +8659,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-16 22:41:48 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6421,7 +6421,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8612,7 +8612,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8659,7 +8659,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-17 12:53:48 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6421,7 +6421,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8612,7 +8612,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8659,7 +8659,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-17 14:47:05 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6421,7 +6421,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8612,7 +8612,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8659,7 +8659,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-17 19:15:07 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6421,7 +6421,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8612,7 +8612,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8659,7 +8659,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-17 22:26:06 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6421,7 +6421,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8612,7 +8612,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8659,7 +8659,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-17 23:37:02 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6421,7 +6421,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8612,7 +8612,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8659,7 +8659,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-18 11:13:56 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6421,7 +6421,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8612,7 +8612,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8659,7 +8659,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-18 14:48:05 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6421,7 +6421,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8612,7 +8612,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8659,7 +8659,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-20 05:15:48 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>43.2%</t>
+          <t>43.6%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>65.0%</t>
+          <t>65.2%</t>
         </is>
       </c>
     </row>
@@ -1289,10 +1289,10 @@
         <v>16</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
@@ -1364,22 +1364,22 @@
         <v>50</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P16" s="4" t="n">
         <v>25</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>32.0%</t>
+          <t>34.0%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>69.3%</t>
+          <t>70.0%</t>
         </is>
       </c>
     </row>
@@ -1445,10 +1445,10 @@
         <v>20</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
@@ -1523,10 +1523,10 @@
         <v>29</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q18" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
@@ -1601,10 +1601,10 @@
         <v>27</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
@@ -1752,45 +1752,45 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>20/07/2026</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr"/>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
       <c r="K23" s="1" t="inlineStr">
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -4680,88 +4680,92 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B87" s="2" t="inlineStr">
+      <c r="A87" s="9" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B87" s="9" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C87" s="2" t="inlineStr">
+      <c r="C87" s="9" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D87" s="2" t="inlineStr">
+      <c r="D87" s="9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E87" s="2" t="inlineStr">
+      <c r="E87" s="9" t="inlineStr">
         <is>
           <t>19/07/2026</t>
         </is>
       </c>
-      <c r="F87" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G87" s="2" t="inlineStr"/>
-      <c r="H87" s="2" t="inlineStr">
+      <c r="F87" s="9" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G87" s="9" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="H87" s="9" t="inlineStr">
+        <is>
+          <t>59/73</t>
+        </is>
+      </c>
+      <c r="I87" s="9" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>PSYCHIATRY</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>20/07/2026</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr"/>
+      <c r="H88" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I87" s="2" t="inlineStr">
+      <c r="I88" s="2" t="inlineStr">
         <is>
           <t>Not Recorded</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B88" s="5" t="inlineStr">
-        <is>
-          <t>A2B</t>
-        </is>
-      </c>
-      <c r="C88" s="5" t="inlineStr">
-        <is>
-          <t>PSYCHIATRY</t>
-        </is>
-      </c>
-      <c r="D88" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E88" s="5" t="inlineStr">
-        <is>
-          <t>20/07/2026</t>
-        </is>
-      </c>
-      <c r="F88" s="5" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G88" s="5" t="inlineStr"/>
-      <c r="H88" s="5" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I88" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -6233,7 +6237,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6280,7 +6284,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6327,7 +6331,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6374,7 +6378,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6421,7 +6425,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -6483,45 +6487,45 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B128" s="5" t="inlineStr">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C128" s="5" t="inlineStr">
+      <c r="C128" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D128" s="5" t="inlineStr">
+      <c r="D128" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E128" s="5" t="inlineStr">
+      <c r="E128" s="2" t="inlineStr">
         <is>
           <t>20/07/2026</t>
         </is>
       </c>
-      <c r="F128" s="5" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G128" s="5" t="inlineStr"/>
-      <c r="H128" s="5" t="inlineStr">
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr"/>
+      <c r="H128" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I128" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -7653,45 +7657,45 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B154" s="5" t="inlineStr">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C154" s="5" t="inlineStr">
+      <c r="C154" s="2" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D154" s="5" t="inlineStr">
+      <c r="D154" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E154" s="5" t="inlineStr">
+      <c r="E154" s="2" t="inlineStr">
         <is>
           <t>20/07/2026</t>
         </is>
       </c>
-      <c r="F154" s="5" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G154" s="5" t="inlineStr"/>
-      <c r="H154" s="5" t="inlineStr">
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr"/>
+      <c r="H154" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I154" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -8475,7 +8479,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8522,7 +8526,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8569,7 +8573,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8616,7 +8620,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8663,7 +8667,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">
@@ -10306,45 +10310,45 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="5" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B213" s="5" t="inlineStr">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C213" s="5" t="inlineStr">
+      <c r="C213" s="2" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D213" s="5" t="inlineStr">
+      <c r="D213" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E213" s="5" t="inlineStr">
+      <c r="E213" s="2" t="inlineStr">
         <is>
           <t>20/07/2026</t>
         </is>
       </c>
-      <c r="F213" s="5" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G213" s="5" t="inlineStr"/>
-      <c r="H213" s="5" t="inlineStr">
+      <c r="F213" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G213" s="2" t="inlineStr"/>
+      <c r="H213" s="2" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I213" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I213" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-20 08:36:54 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6237,7 +6237,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6331,7 +6331,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6378,7 +6378,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6425,7 +6425,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8479,7 +8479,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8526,7 +8526,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8573,7 +8573,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8667,7 +8667,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-20 13:37:43 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6241,7 +6241,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6335,7 +6335,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6382,7 +6382,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8487,7 +8487,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8534,7 +8534,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8581,7 +8581,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8628,7 +8628,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8675,7 +8675,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-20 19:05:30 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6241,7 +6241,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6335,7 +6335,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6382,7 +6382,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8487,7 +8487,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8534,7 +8534,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8581,7 +8581,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8628,7 +8628,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8675,7 +8675,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-20 20:31:25 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6241,7 +6241,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6335,7 +6335,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6382,7 +6382,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8487,7 +8487,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8534,7 +8534,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8581,7 +8581,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8628,7 +8628,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8675,7 +8675,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-21 10:51:25 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6241,7 +6241,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6335,7 +6335,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6382,7 +6382,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8487,7 +8487,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8534,7 +8534,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8581,7 +8581,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8628,7 +8628,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8675,7 +8675,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-21 14:46:04 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6245,7 +6245,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6292,7 +6292,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6339,7 +6339,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6386,7 +6386,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8495,7 +8495,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8542,7 +8542,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8589,7 +8589,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8636,7 +8636,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8683,7 +8683,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-21 19:27:34 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6245,7 +6245,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6292,7 +6292,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6339,7 +6339,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6386,7 +6386,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8495,7 +8495,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8542,7 +8542,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8589,7 +8589,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8636,7 +8636,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8683,7 +8683,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-21 22:14:10 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6245,7 +6245,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6292,7 +6292,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6339,7 +6339,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6386,7 +6386,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8495,7 +8495,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8542,7 +8542,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8589,7 +8589,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8636,7 +8636,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8683,7 +8683,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-21 23:41:11 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6245,7 +6245,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6292,7 +6292,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6339,7 +6339,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6386,7 +6386,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8495,7 +8495,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8542,7 +8542,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8589,7 +8589,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8636,7 +8636,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8683,7 +8683,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-22 07:21:46 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -96,10 +96,10 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="8">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9">
@@ -1289,10 +1289,10 @@
         <v>16</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
@@ -1367,10 +1367,10 @@
         <v>19</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
@@ -1445,10 +1445,10 @@
         <v>22</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
@@ -1523,10 +1523,10 @@
         <v>29</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q18" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
@@ -1601,10 +1601,10 @@
         <v>27</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
@@ -1868,45 +1868,45 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>22/07/2026</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr"/>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
@@ -1914,7 +1914,7 @@
           <t>Not Recorded</t>
         </is>
       </c>
-      <c r="L25" s="7" t="inlineStr">
+      <c r="L25" s="6" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -1926,43 +1926,43 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>DERMATOLOGY</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D26" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
+      <c r="E26" s="7" t="inlineStr">
         <is>
           <t>23/07/2026</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr"/>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr"/>
+      <c r="H26" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr">
+      <c r="I26" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2908,215 +2908,215 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B47" s="6" t="inlineStr">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C47" s="6" t="inlineStr">
+      <c r="C47" s="7" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D47" s="6" t="inlineStr">
+      <c r="D47" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E47" s="6" t="inlineStr">
+      <c r="E47" s="7" t="inlineStr">
         <is>
           <t>26/07/2026</t>
         </is>
       </c>
-      <c r="F47" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G47" s="6" t="inlineStr"/>
-      <c r="H47" s="6" t="inlineStr">
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr"/>
+      <c r="H47" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I47" s="6" t="inlineStr">
+      <c r="I47" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B48" s="6" t="inlineStr">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C48" s="6" t="inlineStr">
+      <c r="C48" s="7" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D48" s="6" t="inlineStr">
+      <c r="D48" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E48" s="6" t="inlineStr">
+      <c r="E48" s="7" t="inlineStr">
         <is>
           <t>27/07/2026</t>
         </is>
       </c>
-      <c r="F48" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G48" s="6" t="inlineStr"/>
-      <c r="H48" s="6" t="inlineStr">
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr"/>
+      <c r="H48" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I48" s="6" t="inlineStr">
+      <c r="I48" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B49" s="6" t="inlineStr">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C49" s="6" t="inlineStr">
+      <c r="C49" s="7" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
+      <c r="D49" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E49" s="6" t="inlineStr">
+      <c r="E49" s="7" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="F49" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G49" s="6" t="inlineStr"/>
-      <c r="H49" s="6" t="inlineStr">
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr"/>
+      <c r="H49" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I49" s="6" t="inlineStr">
+      <c r="I49" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C50" s="6" t="inlineStr">
+      <c r="C50" s="7" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D50" s="6" t="inlineStr">
+      <c r="D50" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="E50" s="7" t="inlineStr">
         <is>
           <t>29/07/2026</t>
         </is>
       </c>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G50" s="6" t="inlineStr"/>
-      <c r="H50" s="6" t="inlineStr">
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr"/>
+      <c r="H50" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I50" s="6" t="inlineStr">
+      <c r="I50" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C51" s="6" t="inlineStr">
+      <c r="C51" s="7" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D51" s="6" t="inlineStr">
+      <c r="D51" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E51" s="6" t="inlineStr">
+      <c r="E51" s="7" t="inlineStr">
         <is>
           <t>30/07/2026</t>
         </is>
       </c>
-      <c r="F51" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G51" s="6" t="inlineStr"/>
-      <c r="H51" s="6" t="inlineStr">
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr"/>
+      <c r="H51" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I51" s="6" t="inlineStr">
+      <c r="I51" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -4821,301 +4821,301 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B90" s="6" t="inlineStr">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C90" s="6" t="inlineStr">
+      <c r="C90" s="2" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D90" s="6" t="inlineStr">
+      <c r="D90" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E90" s="6" t="inlineStr">
+      <c r="E90" s="2" t="inlineStr">
         <is>
           <t>22/07/2026</t>
         </is>
       </c>
-      <c r="F90" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G90" s="6" t="inlineStr"/>
-      <c r="H90" s="6" t="inlineStr">
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr"/>
+      <c r="H90" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I90" s="6" t="inlineStr">
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>A2B</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>PSYCHIATRY</t>
+        </is>
+      </c>
+      <c r="D91" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="inlineStr">
+        <is>
+          <t>23/07/2026</t>
+        </is>
+      </c>
+      <c r="F91" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G91" s="7" t="inlineStr"/>
+      <c r="H91" s="7" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I91" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B91" s="6" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B92" s="7" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C91" s="6" t="inlineStr">
+      <c r="C92" s="7" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D91" s="6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E91" s="6" t="inlineStr">
-        <is>
-          <t>23/07/2026</t>
-        </is>
-      </c>
-      <c r="F91" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G91" s="6" t="inlineStr"/>
-      <c r="H91" s="6" t="inlineStr">
+      <c r="D92" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="F92" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G92" s="7" t="inlineStr"/>
+      <c r="H92" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I91" s="6" t="inlineStr">
+      <c r="I92" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B92" s="6" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C92" s="6" t="inlineStr">
+      <c r="C93" s="7" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D92" s="6" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E92" s="6" t="inlineStr">
-        <is>
-          <t>26/07/2026</t>
-        </is>
-      </c>
-      <c r="F92" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G92" s="6" t="inlineStr"/>
-      <c r="H92" s="6" t="inlineStr">
+      <c r="D93" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="inlineStr">
+        <is>
+          <t>27/07/2026</t>
+        </is>
+      </c>
+      <c r="F93" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G93" s="7" t="inlineStr"/>
+      <c r="H93" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I92" s="6" t="inlineStr">
+      <c r="I93" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B93" s="6" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C93" s="6" t="inlineStr">
+      <c r="C94" s="7" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D93" s="6" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E93" s="6" t="inlineStr">
-        <is>
-          <t>27/07/2026</t>
-        </is>
-      </c>
-      <c r="F93" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G93" s="6" t="inlineStr"/>
-      <c r="H93" s="6" t="inlineStr">
+      <c r="D94" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E94" s="7" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="F94" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G94" s="7" t="inlineStr"/>
+      <c r="H94" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I93" s="6" t="inlineStr">
+      <c r="I94" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B94" s="6" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C94" s="6" t="inlineStr">
+      <c r="C95" s="7" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D94" s="6" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E94" s="6" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="F94" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G94" s="6" t="inlineStr"/>
-      <c r="H94" s="6" t="inlineStr">
+      <c r="D95" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G95" s="7" t="inlineStr"/>
+      <c r="H95" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I94" s="6" t="inlineStr">
+      <c r="I95" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B95" s="6" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B96" s="7" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C95" s="6" t="inlineStr">
+      <c r="C96" s="7" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D95" s="6" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E95" s="6" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="F95" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G95" s="6" t="inlineStr"/>
-      <c r="H95" s="6" t="inlineStr">
+      <c r="D96" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="F96" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G96" s="7" t="inlineStr"/>
+      <c r="H96" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I95" s="6" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B96" s="6" t="inlineStr">
-        <is>
-          <t>A2B</t>
-        </is>
-      </c>
-      <c r="C96" s="6" t="inlineStr">
-        <is>
-          <t>PSYCHIATRY</t>
-        </is>
-      </c>
-      <c r="D96" s="6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E96" s="6" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="F96" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G96" s="6" t="inlineStr"/>
-      <c r="H96" s="6" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I96" s="6" t="inlineStr">
+      <c r="I96" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -6589,301 +6589,301 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B130" s="6" t="inlineStr">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C130" s="6" t="inlineStr">
+      <c r="C130" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D130" s="6" t="inlineStr">
+      <c r="D130" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E130" s="6" t="inlineStr">
+      <c r="E130" s="2" t="inlineStr">
         <is>
           <t>22/07/2026</t>
         </is>
       </c>
-      <c r="F130" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G130" s="6" t="inlineStr"/>
-      <c r="H130" s="6" t="inlineStr">
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr"/>
+      <c r="H130" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I130" s="6" t="inlineStr">
+      <c r="I130" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B131" s="7" t="inlineStr">
+        <is>
+          <t>A2C</t>
+        </is>
+      </c>
+      <c r="C131" s="7" t="inlineStr">
+        <is>
+          <t>IMMUNOLOGY/HAEMATOLOGY</t>
+        </is>
+      </c>
+      <c r="D131" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E131" s="7" t="inlineStr">
+        <is>
+          <t>23/07/2026</t>
+        </is>
+      </c>
+      <c r="F131" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G131" s="7" t="inlineStr"/>
+      <c r="H131" s="7" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I131" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B131" s="6" t="inlineStr">
+    <row r="132">
+      <c r="A132" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B132" s="7" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C131" s="6" t="inlineStr">
+      <c r="C132" s="7" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D131" s="6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E131" s="6" t="inlineStr">
-        <is>
-          <t>23/07/2026</t>
-        </is>
-      </c>
-      <c r="F131" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G131" s="6" t="inlineStr"/>
-      <c r="H131" s="6" t="inlineStr">
+      <c r="D132" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E132" s="7" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="F132" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G132" s="7" t="inlineStr"/>
+      <c r="H132" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I131" s="6" t="inlineStr">
+      <c r="I132" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="132">
-      <c r="A132" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B132" s="6" t="inlineStr">
+    <row r="133">
+      <c r="A133" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B133" s="7" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C132" s="6" t="inlineStr">
+      <c r="C133" s="7" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D132" s="6" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E132" s="6" t="inlineStr">
-        <is>
-          <t>26/07/2026</t>
-        </is>
-      </c>
-      <c r="F132" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G132" s="6" t="inlineStr"/>
-      <c r="H132" s="6" t="inlineStr">
+      <c r="D133" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E133" s="7" t="inlineStr">
+        <is>
+          <t>27/07/2026</t>
+        </is>
+      </c>
+      <c r="F133" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G133" s="7" t="inlineStr"/>
+      <c r="H133" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I132" s="6" t="inlineStr">
+      <c r="I133" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="133">
-      <c r="A133" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B133" s="6" t="inlineStr">
+    <row r="134">
+      <c r="A134" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B134" s="7" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C133" s="6" t="inlineStr">
+      <c r="C134" s="7" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D133" s="6" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E133" s="6" t="inlineStr">
-        <is>
-          <t>27/07/2026</t>
-        </is>
-      </c>
-      <c r="F133" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G133" s="6" t="inlineStr"/>
-      <c r="H133" s="6" t="inlineStr">
+      <c r="D134" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E134" s="7" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="F134" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G134" s="7" t="inlineStr"/>
+      <c r="H134" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I133" s="6" t="inlineStr">
+      <c r="I134" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B134" s="6" t="inlineStr">
+    <row r="135">
+      <c r="A135" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B135" s="7" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C134" s="6" t="inlineStr">
+      <c r="C135" s="7" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D134" s="6" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E134" s="6" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="F134" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G134" s="6" t="inlineStr"/>
-      <c r="H134" s="6" t="inlineStr">
+      <c r="D135" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E135" s="7" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
+      <c r="F135" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G135" s="7" t="inlineStr"/>
+      <c r="H135" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I134" s="6" t="inlineStr">
+      <c r="I135" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="135">
-      <c r="A135" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B135" s="6" t="inlineStr">
+    <row r="136">
+      <c r="A136" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B136" s="7" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C135" s="6" t="inlineStr">
+      <c r="C136" s="7" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D135" s="6" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E135" s="6" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="F135" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G135" s="6" t="inlineStr"/>
-      <c r="H135" s="6" t="inlineStr">
+      <c r="D136" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E136" s="7" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="F136" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G136" s="7" t="inlineStr"/>
+      <c r="H136" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I135" s="6" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B136" s="6" t="inlineStr">
-        <is>
-          <t>A2C</t>
-        </is>
-      </c>
-      <c r="C136" s="6" t="inlineStr">
-        <is>
-          <t>IMMUNOLOGY/HAEMATOLOGY</t>
-        </is>
-      </c>
-      <c r="D136" s="6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E136" s="6" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="F136" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G136" s="6" t="inlineStr"/>
-      <c r="H136" s="6" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I136" s="6" t="inlineStr">
+      <c r="I136" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -7759,258 +7759,258 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B156" s="6" t="inlineStr">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C156" s="6" t="inlineStr">
+      <c r="C156" s="2" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D156" s="6" t="inlineStr">
+      <c r="D156" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E156" s="6" t="inlineStr">
+      <c r="E156" s="2" t="inlineStr">
         <is>
           <t>22/07/2026</t>
         </is>
       </c>
-      <c r="F156" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G156" s="6" t="inlineStr"/>
-      <c r="H156" s="6" t="inlineStr">
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="inlineStr"/>
+      <c r="H156" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I156" s="6" t="inlineStr">
+      <c r="I156" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B157" s="7" t="inlineStr">
+        <is>
+          <t>A2D</t>
+        </is>
+      </c>
+      <c r="C157" s="7" t="inlineStr">
+        <is>
+          <t>CARDIOLOGY</t>
+        </is>
+      </c>
+      <c r="D157" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E157" s="7" t="inlineStr">
+        <is>
+          <t>25/07/2026</t>
+        </is>
+      </c>
+      <c r="F157" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G157" s="7" t="inlineStr"/>
+      <c r="H157" s="7" t="inlineStr">
+        <is>
+          <t>0/73</t>
+        </is>
+      </c>
+      <c r="I157" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="157">
-      <c r="A157" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B157" s="6" t="inlineStr">
+    <row r="158">
+      <c r="A158" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B158" s="7" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C157" s="6" t="inlineStr">
+      <c r="C158" s="7" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D157" s="6" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E157" s="6" t="inlineStr">
-        <is>
-          <t>25/07/2026</t>
-        </is>
-      </c>
-      <c r="F157" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G157" s="6" t="inlineStr"/>
-      <c r="H157" s="6" t="inlineStr">
+      <c r="D158" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E158" s="7" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="F158" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G158" s="7" t="inlineStr"/>
+      <c r="H158" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I157" s="6" t="inlineStr">
+      <c r="I158" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="158">
-      <c r="A158" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B158" s="6" t="inlineStr">
+    <row r="159">
+      <c r="A159" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B159" s="7" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C158" s="6" t="inlineStr">
+      <c r="C159" s="7" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D158" s="6" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E158" s="6" t="inlineStr">
-        <is>
-          <t>26/07/2026</t>
-        </is>
-      </c>
-      <c r="F158" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G158" s="6" t="inlineStr"/>
-      <c r="H158" s="6" t="inlineStr">
+      <c r="D159" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E159" s="7" t="inlineStr">
+        <is>
+          <t>27/07/2026</t>
+        </is>
+      </c>
+      <c r="F159" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G159" s="7" t="inlineStr"/>
+      <c r="H159" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I158" s="6" t="inlineStr">
+      <c r="I159" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="159">
-      <c r="A159" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B159" s="6" t="inlineStr">
+    <row r="160">
+      <c r="A160" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B160" s="7" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C159" s="6" t="inlineStr">
+      <c r="C160" s="7" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D159" s="6" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E159" s="6" t="inlineStr">
-        <is>
-          <t>27/07/2026</t>
-        </is>
-      </c>
-      <c r="F159" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G159" s="6" t="inlineStr"/>
-      <c r="H159" s="6" t="inlineStr">
+      <c r="D160" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E160" s="7" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="F160" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G160" s="7" t="inlineStr"/>
+      <c r="H160" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I159" s="6" t="inlineStr">
+      <c r="I160" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="160">
-      <c r="A160" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B160" s="6" t="inlineStr">
+    <row r="161">
+      <c r="A161" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B161" s="7" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C160" s="6" t="inlineStr">
+      <c r="C161" s="7" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D160" s="6" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E160" s="6" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="F160" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G160" s="6" t="inlineStr"/>
-      <c r="H160" s="6" t="inlineStr">
+      <c r="D161" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E161" s="7" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
+      <c r="F161" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G161" s="7" t="inlineStr"/>
+      <c r="H161" s="7" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I160" s="6" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B161" s="6" t="inlineStr">
-        <is>
-          <t>A2D</t>
-        </is>
-      </c>
-      <c r="C161" s="6" t="inlineStr">
-        <is>
-          <t>CARDIOLOGY</t>
-        </is>
-      </c>
-      <c r="D161" s="6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E161" s="6" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="F161" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G161" s="6" t="inlineStr"/>
-      <c r="H161" s="6" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I161" s="6" t="inlineStr">
+      <c r="I161" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -10412,301 +10412,301 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B215" s="6" t="inlineStr">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C215" s="6" t="inlineStr">
+      <c r="C215" s="2" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D215" s="6" t="inlineStr">
+      <c r="D215" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E215" s="6" t="inlineStr">
+      <c r="E215" s="2" t="inlineStr">
         <is>
           <t>22/07/2026</t>
         </is>
       </c>
-      <c r="F215" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G215" s="6" t="inlineStr"/>
-      <c r="H215" s="6" t="inlineStr">
+      <c r="F215" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G215" s="2" t="inlineStr"/>
+      <c r="H215" s="2" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I215" s="6" t="inlineStr">
+      <c r="I215" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B216" s="7" t="inlineStr">
+        <is>
+          <t>A2E</t>
+        </is>
+      </c>
+      <c r="C216" s="7" t="inlineStr">
+        <is>
+          <t>CHEST</t>
+        </is>
+      </c>
+      <c r="D216" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E216" s="7" t="inlineStr">
+        <is>
+          <t>23/07/2026</t>
+        </is>
+      </c>
+      <c r="F216" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G216" s="7" t="inlineStr"/>
+      <c r="H216" s="7" t="inlineStr">
+        <is>
+          <t>0/37</t>
+        </is>
+      </c>
+      <c r="I216" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="216">
-      <c r="A216" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B216" s="6" t="inlineStr">
+    <row r="217">
+      <c r="A217" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B217" s="7" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C216" s="6" t="inlineStr">
+      <c r="C217" s="7" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D216" s="6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E216" s="6" t="inlineStr">
-        <is>
-          <t>23/07/2026</t>
-        </is>
-      </c>
-      <c r="F216" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G216" s="6" t="inlineStr"/>
-      <c r="H216" s="6" t="inlineStr">
+      <c r="D217" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E217" s="7" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="F217" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G217" s="7" t="inlineStr"/>
+      <c r="H217" s="7" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I216" s="6" t="inlineStr">
+      <c r="I217" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="217">
-      <c r="A217" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B217" s="6" t="inlineStr">
+    <row r="218">
+      <c r="A218" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B218" s="7" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C217" s="6" t="inlineStr">
+      <c r="C218" s="7" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D217" s="6" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E217" s="6" t="inlineStr">
-        <is>
-          <t>26/07/2026</t>
-        </is>
-      </c>
-      <c r="F217" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G217" s="6" t="inlineStr"/>
-      <c r="H217" s="6" t="inlineStr">
+      <c r="D218" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E218" s="7" t="inlineStr">
+        <is>
+          <t>27/07/2026</t>
+        </is>
+      </c>
+      <c r="F218" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G218" s="7" t="inlineStr"/>
+      <c r="H218" s="7" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I217" s="6" t="inlineStr">
+      <c r="I218" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="218">
-      <c r="A218" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B218" s="6" t="inlineStr">
+    <row r="219">
+      <c r="A219" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B219" s="7" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C218" s="6" t="inlineStr">
+      <c r="C219" s="7" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D218" s="6" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E218" s="6" t="inlineStr">
-        <is>
-          <t>27/07/2026</t>
-        </is>
-      </c>
-      <c r="F218" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G218" s="6" t="inlineStr"/>
-      <c r="H218" s="6" t="inlineStr">
+      <c r="D219" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E219" s="7" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="F219" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G219" s="7" t="inlineStr"/>
+      <c r="H219" s="7" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I218" s="6" t="inlineStr">
+      <c r="I219" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="219">
-      <c r="A219" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B219" s="6" t="inlineStr">
+    <row r="220">
+      <c r="A220" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B220" s="7" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C219" s="6" t="inlineStr">
+      <c r="C220" s="7" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D219" s="6" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E219" s="6" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="F219" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G219" s="6" t="inlineStr"/>
-      <c r="H219" s="6" t="inlineStr">
+      <c r="D220" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E220" s="7" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
+      <c r="F220" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G220" s="7" t="inlineStr"/>
+      <c r="H220" s="7" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I219" s="6" t="inlineStr">
+      <c r="I220" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="220">
-      <c r="A220" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B220" s="6" t="inlineStr">
+    <row r="221">
+      <c r="A221" s="7" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B221" s="7" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C220" s="6" t="inlineStr">
+      <c r="C221" s="7" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D220" s="6" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E220" s="6" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="F220" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G220" s="6" t="inlineStr"/>
-      <c r="H220" s="6" t="inlineStr">
+      <c r="D221" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E221" s="7" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="F221" s="7" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G221" s="7" t="inlineStr"/>
+      <c r="H221" s="7" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I220" s="6" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B221" s="6" t="inlineStr">
-        <is>
-          <t>A2E</t>
-        </is>
-      </c>
-      <c r="C221" s="6" t="inlineStr">
-        <is>
-          <t>CHEST</t>
-        </is>
-      </c>
-      <c r="D221" s="6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E221" s="6" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
-      <c r="F221" s="6" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G221" s="6" t="inlineStr"/>
-      <c r="H221" s="6" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I221" s="6" t="inlineStr">
+      <c r="I221" s="7" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-22 13:51:32 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6249,7 +6249,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6437,7 +6437,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8503,7 +8503,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8550,7 +8550,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8597,7 +8597,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-23 03:30:58 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
@@ -6249,7 +6249,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="9" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="9" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="9" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="9" t="inlineStr">
@@ -6437,7 +6437,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="9" t="inlineStr">
@@ -8503,7 +8503,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -8550,7 +8550,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="9" t="inlineStr">
@@ -8597,7 +8597,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="9" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="9" t="inlineStr">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-23 09:16:22 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
@@ -6249,7 +6249,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="8" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="8" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
@@ -6437,7 +6437,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="8" t="inlineStr">
@@ -8503,7 +8503,7 @@
       </c>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="8" t="inlineStr">
@@ -8550,7 +8550,7 @@
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="8" t="inlineStr">
@@ -8597,7 +8597,7 @@
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="8" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="8" t="inlineStr">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-23 18:24:17 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
@@ -6249,7 +6249,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="8" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="8" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
@@ -6437,7 +6437,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="8" t="inlineStr">
@@ -8503,7 +8503,7 @@
       </c>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="8" t="inlineStr">
@@ -8550,7 +8550,7 @@
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="8" t="inlineStr">
@@ -8597,7 +8597,7 @@
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="8" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="8" t="inlineStr">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-24 01:08:54 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
@@ -6249,7 +6249,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="8" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="8" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
@@ -6437,7 +6437,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="8" t="inlineStr">
@@ -8503,7 +8503,7 @@
       </c>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="8" t="inlineStr">
@@ -8550,7 +8550,7 @@
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="8" t="inlineStr">
@@ -8597,7 +8597,7 @@
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="8" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="8" t="inlineStr">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-24 15:27:16 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
@@ -6249,7 +6249,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="8" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="8" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
@@ -6437,7 +6437,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="8" t="inlineStr">
@@ -8503,7 +8503,7 @@
       </c>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="8" t="inlineStr">
@@ -8550,7 +8550,7 @@
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="8" t="inlineStr">
@@ -8597,7 +8597,7 @@
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="8" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="8" t="inlineStr">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-25 03:59:53 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
@@ -6249,7 +6249,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="8" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="8" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
@@ -6437,7 +6437,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="8" t="inlineStr">
@@ -8503,7 +8503,7 @@
       </c>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="8" t="inlineStr">
@@ -8550,7 +8550,7 @@
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="8" t="inlineStr">
@@ -8597,7 +8597,7 @@
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="8" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="8" t="inlineStr">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-25 08:42:06 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
@@ -6249,7 +6249,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="8" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="8" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
@@ -6437,7 +6437,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="8" t="inlineStr">
@@ -8503,7 +8503,7 @@
       </c>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="8" t="inlineStr">
@@ -8550,7 +8550,7 @@
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="8" t="inlineStr">
@@ -8597,7 +8597,7 @@
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="8" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="8" t="inlineStr">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-25 14:59:20 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
@@ -6249,7 +6249,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="8" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="8" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
@@ -6437,7 +6437,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="8" t="inlineStr">
@@ -8503,7 +8503,7 @@
       </c>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="8" t="inlineStr">
@@ -8550,7 +8550,7 @@
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="8" t="inlineStr">
@@ -8597,7 +8597,7 @@
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="8" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="8" t="inlineStr">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-25 16:13:48 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
@@ -6249,7 +6249,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="8" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="8" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
@@ -6437,7 +6437,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="8" t="inlineStr">
@@ -8503,7 +8503,7 @@
       </c>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="8" t="inlineStr">
@@ -8550,7 +8550,7 @@
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="8" t="inlineStr">
@@ -8597,7 +8597,7 @@
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="8" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="8" t="inlineStr">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-25 18:41:43 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
@@ -6249,7 +6249,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="8" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="8" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
@@ -6437,7 +6437,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="8" t="inlineStr">
@@ -8503,7 +8503,7 @@
       </c>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="8" t="inlineStr">
@@ -8550,7 +8550,7 @@
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="8" t="inlineStr">
@@ -8597,7 +8597,7 @@
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="8" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="8" t="inlineStr">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-26 06:10:22 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9">
@@ -1289,10 +1289,10 @@
         <v>16</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
@@ -1367,10 +1367,10 @@
         <v>20</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
@@ -1445,10 +1445,10 @@
         <v>23</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
@@ -1523,10 +1523,10 @@
         <v>29</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="Q18" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
@@ -1601,10 +1601,10 @@
         <v>27</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
@@ -2908,45 +2908,45 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B47" s="9" t="inlineStr">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C47" s="9" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D47" s="9" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E47" s="9" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>26/07/2026</t>
         </is>
       </c>
-      <c r="F47" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G47" s="9" t="inlineStr"/>
-      <c r="H47" s="9" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I47" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -4911,45 +4911,45 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B92" s="9" t="inlineStr">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C92" s="9" t="inlineStr">
+      <c r="C92" s="2" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D92" s="9" t="inlineStr">
+      <c r="D92" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E92" s="9" t="inlineStr">
+      <c r="E92" s="2" t="inlineStr">
         <is>
           <t>26/07/2026</t>
         </is>
       </c>
-      <c r="F92" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G92" s="9" t="inlineStr"/>
-      <c r="H92" s="9" t="inlineStr">
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr"/>
+      <c r="H92" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I92" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -6683,45 +6683,45 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B132" s="9" t="inlineStr">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C132" s="9" t="inlineStr">
+      <c r="C132" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D132" s="9" t="inlineStr">
+      <c r="D132" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E132" s="9" t="inlineStr">
+      <c r="E132" s="2" t="inlineStr">
         <is>
           <t>26/07/2026</t>
         </is>
       </c>
-      <c r="F132" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G132" s="9" t="inlineStr"/>
-      <c r="H132" s="9" t="inlineStr">
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr"/>
+      <c r="H132" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I132" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -7853,45 +7853,45 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B158" s="9" t="inlineStr">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C158" s="9" t="inlineStr">
+      <c r="C158" s="2" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D158" s="9" t="inlineStr">
+      <c r="D158" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E158" s="9" t="inlineStr">
+      <c r="E158" s="2" t="inlineStr">
         <is>
           <t>26/07/2026</t>
         </is>
       </c>
-      <c r="F158" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G158" s="9" t="inlineStr"/>
-      <c r="H158" s="9" t="inlineStr">
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G158" s="2" t="inlineStr"/>
+      <c r="H158" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I158" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I158" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -10506,45 +10506,45 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B217" s="9" t="inlineStr">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C217" s="9" t="inlineStr">
+      <c r="C217" s="2" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D217" s="9" t="inlineStr">
+      <c r="D217" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E217" s="9" t="inlineStr">
+      <c r="E217" s="2" t="inlineStr">
         <is>
           <t>26/07/2026</t>
         </is>
       </c>
-      <c r="F217" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G217" s="9" t="inlineStr"/>
-      <c r="H217" s="9" t="inlineStr">
+      <c r="F217" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G217" s="2" t="inlineStr"/>
+      <c r="H217" s="2" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I217" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I217" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-26 11:57:57 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>46.0%</t>
+          <t>46.8%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>65.2%</t>
+          <t>65.0%</t>
         </is>
       </c>
     </row>
@@ -1364,22 +1364,22 @@
         <v>50</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>42.0%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>71.7%</t>
+          <t>71.6%</t>
         </is>
       </c>
     </row>
@@ -1442,22 +1442,22 @@
         <v>50</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>46.0%</t>
+          <t>48.0%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>77.8%</t>
+          <t>76.4%</t>
         </is>
       </c>
     </row>
@@ -4911,45 +4911,49 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B92" s="2" t="inlineStr">
+      <c r="A92" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B92" s="8" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C92" s="2" t="inlineStr">
+      <c r="C92" s="8" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D92" s="2" t="inlineStr">
+      <c r="D92" s="8" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E92" s="2" t="inlineStr">
+      <c r="E92" s="8" t="inlineStr">
         <is>
           <t>26/07/2026</t>
         </is>
       </c>
-      <c r="F92" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G92" s="2" t="inlineStr"/>
-      <c r="H92" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I92" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F92" s="8" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G92" s="8" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H92" s="8" t="inlineStr">
+        <is>
+          <t>50/73</t>
+        </is>
+      </c>
+      <c r="I92" s="8" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -6683,45 +6687,49 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B132" s="2" t="inlineStr">
+      <c r="A132" s="8" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B132" s="8" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C132" s="2" t="inlineStr">
+      <c r="C132" s="8" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D132" s="2" t="inlineStr">
+      <c r="D132" s="8" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E132" s="2" t="inlineStr">
+      <c r="E132" s="8" t="inlineStr">
         <is>
           <t>26/07/2026</t>
         </is>
       </c>
-      <c r="F132" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G132" s="2" t="inlineStr"/>
-      <c r="H132" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I132" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F132" s="8" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G132" s="8" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H132" s="8" t="inlineStr">
+        <is>
+          <t>31/73</t>
+        </is>
+      </c>
+      <c r="I132" s="8" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-26 16:12:41 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4015,7 +4015,7 @@
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="8" t="inlineStr">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="8" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
@@ -6253,7 +6253,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="8" t="inlineStr">
@@ -6300,7 +6300,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="8" t="inlineStr">
@@ -6347,7 +6347,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="8" t="inlineStr">
@@ -6394,7 +6394,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="8" t="inlineStr">
@@ -6441,7 +6441,7 @@
       </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="8" t="inlineStr">
@@ -8511,7 +8511,7 @@
       </c>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="8" t="inlineStr">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="8" t="inlineStr">
@@ -8605,7 +8605,7 @@
       </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="8" t="inlineStr">
@@ -8652,7 +8652,7 @@
       </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="8" t="inlineStr">
@@ -8699,7 +8699,7 @@
       </c>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-27 05:21:52 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>114</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -1289,10 +1289,10 @@
         <v>16</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
@@ -1367,10 +1367,10 @@
         <v>21</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
@@ -1445,10 +1445,10 @@
         <v>24</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
@@ -1523,10 +1523,10 @@
         <v>29</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q18" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
@@ -1601,10 +1601,10 @@
         <v>27</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
@@ -2951,45 +2951,45 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B48" s="9" t="inlineStr">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C48" s="9" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D48" s="9" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E48" s="9" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>27/07/2026</t>
         </is>
       </c>
-      <c r="F48" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G48" s="9" t="inlineStr"/>
-      <c r="H48" s="9" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I48" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -4958,45 +4958,45 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B93" s="9" t="inlineStr">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C93" s="9" t="inlineStr">
+      <c r="C93" s="2" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D93" s="9" t="inlineStr">
+      <c r="D93" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E93" s="9" t="inlineStr">
+      <c r="E93" s="2" t="inlineStr">
         <is>
           <t>27/07/2026</t>
         </is>
       </c>
-      <c r="F93" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G93" s="9" t="inlineStr"/>
-      <c r="H93" s="9" t="inlineStr">
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr"/>
+      <c r="H93" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I93" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -6734,45 +6734,45 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B133" s="9" t="inlineStr">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C133" s="9" t="inlineStr">
+      <c r="C133" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D133" s="9" t="inlineStr">
+      <c r="D133" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E133" s="9" t="inlineStr">
+      <c r="E133" s="2" t="inlineStr">
         <is>
           <t>27/07/2026</t>
         </is>
       </c>
-      <c r="F133" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G133" s="9" t="inlineStr"/>
-      <c r="H133" s="9" t="inlineStr">
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr"/>
+      <c r="H133" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I133" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I133" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -7904,45 +7904,45 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B159" s="9" t="inlineStr">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C159" s="9" t="inlineStr">
+      <c r="C159" s="2" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D159" s="9" t="inlineStr">
+      <c r="D159" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E159" s="9" t="inlineStr">
+      <c r="E159" s="2" t="inlineStr">
         <is>
           <t>27/07/2026</t>
         </is>
       </c>
-      <c r="F159" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G159" s="9" t="inlineStr"/>
-      <c r="H159" s="9" t="inlineStr">
+      <c r="F159" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G159" s="2" t="inlineStr"/>
+      <c r="H159" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I159" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I159" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -10557,45 +10557,45 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B218" s="9" t="inlineStr">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C218" s="9" t="inlineStr">
+      <c r="C218" s="2" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D218" s="9" t="inlineStr">
+      <c r="D218" s="2" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E218" s="9" t="inlineStr">
+      <c r="E218" s="2" t="inlineStr">
         <is>
           <t>27/07/2026</t>
         </is>
       </c>
-      <c r="F218" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G218" s="9" t="inlineStr"/>
-      <c r="H218" s="9" t="inlineStr">
+      <c r="F218" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G218" s="2" t="inlineStr"/>
+      <c r="H218" s="2" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I218" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I218" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-28 06:31:26 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -1305,10 +1305,10 @@
         <v>31</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
@@ -1387,10 +1387,10 @@
         <v>31</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
@@ -1469,10 +1469,10 @@
         <v>24</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
@@ -1551,10 +1551,10 @@
         <v>29</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q18" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
@@ -1633,10 +1633,10 @@
         <v>27</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
@@ -3054,45 +3054,45 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B49" s="9" t="inlineStr">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C49" s="9" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D49" s="9" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E49" s="9" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="F49" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G49" s="9" t="inlineStr"/>
-      <c r="H49" s="9" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr"/>
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I49" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -5101,45 +5101,45 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B94" s="9" t="inlineStr">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C94" s="9" t="inlineStr">
+      <c r="C94" s="2" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D94" s="9" t="inlineStr">
+      <c r="D94" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E94" s="9" t="inlineStr">
+      <c r="E94" s="2" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="F94" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G94" s="9" t="inlineStr"/>
-      <c r="H94" s="9" t="inlineStr">
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr"/>
+      <c r="H94" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I94" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -6877,45 +6877,45 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B134" s="9" t="inlineStr">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C134" s="9" t="inlineStr">
+      <c r="C134" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D134" s="9" t="inlineStr">
+      <c r="D134" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E134" s="9" t="inlineStr">
+      <c r="E134" s="2" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="F134" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G134" s="9" t="inlineStr"/>
-      <c r="H134" s="9" t="inlineStr">
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr"/>
+      <c r="H134" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I134" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -8047,45 +8047,45 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B160" s="9" t="inlineStr">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
         <is>
           <t>A2D</t>
         </is>
       </c>
-      <c r="C160" s="9" t="inlineStr">
+      <c r="C160" s="2" t="inlineStr">
         <is>
           <t>CARDIOLOGY</t>
         </is>
       </c>
-      <c r="D160" s="9" t="inlineStr">
+      <c r="D160" s="2" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E160" s="9" t="inlineStr">
+      <c r="E160" s="2" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="F160" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G160" s="9" t="inlineStr"/>
-      <c r="H160" s="9" t="inlineStr">
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G160" s="2" t="inlineStr"/>
+      <c r="H160" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I160" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I160" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -10700,45 +10700,45 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B219" s="9" t="inlineStr">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C219" s="9" t="inlineStr">
+      <c r="C219" s="2" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D219" s="9" t="inlineStr">
+      <c r="D219" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E219" s="9" t="inlineStr">
+      <c r="E219" s="2" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="F219" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G219" s="9" t="inlineStr"/>
-      <c r="H219" s="9" t="inlineStr">
+      <c r="F219" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G219" s="2" t="inlineStr"/>
+      <c r="H219" s="2" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I219" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I219" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-28 09:23:31 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>56.8%</t>
+          <t>57.6%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>68.5%</t>
+          <t>68.2%</t>
         </is>
       </c>
     </row>
@@ -1302,22 +1302,22 @@
         <v>50</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>2</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>62.0%</t>
+          <t>64.0%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>75.7%</t>
+          <t>75.1%</t>
         </is>
       </c>
     </row>
@@ -1466,22 +1466,22 @@
         <v>50</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>2</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>48.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>76.4%</t>
+          <t>75.0%</t>
         </is>
       </c>
     </row>
@@ -3054,45 +3054,49 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D49" s="5" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="E49" s="5" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G49" s="2" t="inlineStr"/>
-      <c r="H49" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I49" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>40/73</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -6834,45 +6838,49 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B133" s="2" t="inlineStr">
+      <c r="A133" s="5" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C133" s="2" t="inlineStr">
+      <c r="C133" s="5" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D133" s="2" t="inlineStr">
+      <c r="D133" s="5" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E133" s="2" t="inlineStr">
+      <c r="E133" s="5" t="inlineStr">
         <is>
           <t>27/07/2026</t>
         </is>
       </c>
-      <c r="F133" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G133" s="2" t="inlineStr"/>
-      <c r="H133" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I133" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F133" s="5" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G133" s="5" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H133" s="5" t="inlineStr">
+        <is>
+          <t>30/73</t>
+        </is>
+      </c>
+      <c r="I133" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-28 19:24:35 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4115,7 +4115,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4162,7 +4162,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4209,7 +4209,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4256,7 +4256,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6357,7 +6357,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6404,7 +6404,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6451,7 +6451,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6498,7 +6498,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6545,7 +6545,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8619,7 +8619,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8666,7 +8666,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8713,7 +8713,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8760,7 +8760,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8807,7 +8807,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-29 19:16:58 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>57.6%</t>
+          <t>58.0%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>68.2%</t>
+          <t>68.3%</t>
         </is>
       </c>
     </row>
@@ -1302,22 +1302,22 @@
         <v>50</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>1</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>64.0%</t>
+          <t>66.0%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>75.1%</t>
+          <t>75.4%</t>
         </is>
       </c>
     </row>
@@ -3101,45 +3101,49 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C50" s="5" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="D50" s="5" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E50" s="5" t="inlineStr">
         <is>
           <t>29/07/2026</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="inlineStr"/>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>0/73</t>
-        </is>
-      </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>61/73</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-30 05:23:46 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -81,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -103,9 +103,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -845,7 +842,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8">
@@ -896,7 +893,7 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1305,10 +1302,10 @@
         <v>33</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
@@ -1387,10 +1384,10 @@
         <v>31</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
@@ -1469,10 +1466,10 @@
         <v>25</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
@@ -1633,10 +1630,10 @@
         <v>27</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
@@ -3148,45 +3145,45 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B51" s="9" t="inlineStr">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>A2A</t>
         </is>
       </c>
-      <c r="C51" s="9" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>TROPICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D51" s="9" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E51" s="9" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>30/07/2026</t>
         </is>
       </c>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G51" s="9" t="inlineStr"/>
-      <c r="H51" s="9" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr"/>
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I51" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -5195,45 +5192,45 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B96" s="9" t="inlineStr">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
         <is>
           <t>A2B</t>
         </is>
       </c>
-      <c r="C96" s="9" t="inlineStr">
+      <c r="C96" s="2" t="inlineStr">
         <is>
           <t>PSYCHIATRY</t>
         </is>
       </c>
-      <c r="D96" s="9" t="inlineStr">
+      <c r="D96" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E96" s="9" t="inlineStr">
+      <c r="E96" s="2" t="inlineStr">
         <is>
           <t>30/07/2026</t>
         </is>
       </c>
-      <c r="F96" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G96" s="9" t="inlineStr"/>
-      <c r="H96" s="9" t="inlineStr">
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr"/>
+      <c r="H96" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I96" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -6975,45 +6972,45 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B136" s="9" t="inlineStr">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
         <is>
           <t>A2C</t>
         </is>
       </c>
-      <c r="C136" s="9" t="inlineStr">
+      <c r="C136" s="2" t="inlineStr">
         <is>
           <t>IMMUNOLOGY/HAEMATOLOGY</t>
         </is>
       </c>
-      <c r="D136" s="9" t="inlineStr">
+      <c r="D136" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E136" s="9" t="inlineStr">
+      <c r="E136" s="2" t="inlineStr">
         <is>
           <t>30/07/2026</t>
         </is>
       </c>
-      <c r="F136" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G136" s="9" t="inlineStr"/>
-      <c r="H136" s="9" t="inlineStr">
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr"/>
+      <c r="H136" s="2" t="inlineStr">
         <is>
           <t>0/73</t>
         </is>
       </c>
-      <c r="I136" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I136" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -10798,45 +10795,45 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="9" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B221" s="9" t="inlineStr">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="B221" s="2" t="inlineStr">
         <is>
           <t>A2E</t>
         </is>
       </c>
-      <c r="C221" s="9" t="inlineStr">
+      <c r="C221" s="2" t="inlineStr">
         <is>
           <t>CHEST</t>
         </is>
       </c>
-      <c r="D221" s="9" t="inlineStr">
+      <c r="D221" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E221" s="9" t="inlineStr">
+      <c r="E221" s="2" t="inlineStr">
         <is>
           <t>30/07/2026</t>
         </is>
       </c>
-      <c r="F221" s="9" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G221" s="9" t="inlineStr"/>
-      <c r="H221" s="9" t="inlineStr">
+      <c r="F221" s="2" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G221" s="2" t="inlineStr"/>
+      <c r="H221" s="2" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I221" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I221" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-30 16:31:58 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4116,7 +4116,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4257,7 +4257,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6405,7 +6405,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6452,7 +6452,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6499,7 +6499,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6546,7 +6546,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8667,7 +8667,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8808,7 +8808,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-30 23:40:31 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-31 05:58:32 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-31 17:31:59 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-31 20:26:09 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-31 21:43:30 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-01 15:05:45 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-02 00:02:07 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-02 05:49:07 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-02 10:20:20 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-02 22:00:12 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-03 02:34:18 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-04 08:11:07 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-04 13:23:19 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-04 21:00:01 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-05 11:07:27 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-05 18:46:28 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-06 02:26:50 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-06 15:49:27 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-07 08:00:01 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-07 17:30:00 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-07 21:17:17 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-07 23:11:56 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-08 12:42:52 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-08 16:36:35 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-08 21:03:13 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-08 21:39:06 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-09 17:36:29 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-09 19:35:25 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-09 20:46:13 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-09 22:06:31 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-10 05:30:34 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-10 08:33:32 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-10 10:05:34 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-10 16:59:26 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-10 21:45:25 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-11 04:24:36 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-11 09:38:40 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2024/2025, 2025/2026</t>
+          <t>2025/2026, 2024/2025</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-12 16:35:35 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
+++ b/attendance_reports/Y4_B2526_General_&_Special_Internal_1_A2_session_analysis.xlsx
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="G173" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G174" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="G175" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="G176" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">

</xml_diff>